<commit_message>
Tesis B: rehacer long list con empresas del sector insights (bloques 2 y 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015eGgGxXjnPfmv7TgBdyPpP
</commit_message>
<xml_diff>
--- a/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
+++ b/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>The Cocktail Analysis</t>
+          <t>Instituto DYM</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -711,17 +711,17 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Independiente (spin-off de The Cocktail)</t>
+          <t>Independiente; fundado en 1962</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Consultora de investigación en tendencias de consumo, comunicación y tecnología</t>
+          <t>Instituto full-service ad hoc (cuanti y cuali); 49 empleados en 2024; socio de I+A España</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Entrada en gran consumo y retail con posicionamiento premium cualitativo; mismo perfil consultivo que Psyma</t>
+          <t>Cartera de gran consumo y capacidad de campo; tamaño asumible para una primera compra</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>tca-ss.com</t>
+          <t>institutodym.es</t>
         </is>
       </c>
       <c r="N5" s="6" t="n"/>
@@ -765,12 +765,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Instituto DYM</t>
+          <t>Ikerfel</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Bilbao</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -780,17 +780,17 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Independiente; fundado en 1962</t>
+          <t>Independiente; fundado en 1976</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Instituto full-service ad hoc (cuanti y cuali), ~49 empleados en 2024</t>
+          <t>Investigación de mercados y estrategia; +7.000 estudios; socio de I+A España</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Capacidad de campo y cartera multisector; tamaño digerible para una primera adquisición</t>
+          <t>Cobertura del norte de España; clientes de consumo y utilities</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>institutodym.es</t>
+          <t>ikerfel.es</t>
         </is>
       </c>
       <c r="N6" s="6" t="n"/>
@@ -834,12 +834,12 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Ikerfel</t>
+          <t>More than Research</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Bilbao</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Independiente; fundado en 1976</t>
+          <t>Fundador (ex Infratest, Synovate, Ipsos); fundada en 2011</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Investigación de mercados y estrategia; +7.000 estudios en consumo, servicios y sector público</t>
+          <t>Agencia multidisciplinar: marketing y publicidad, UX, pharma y social media; socio de I+A España</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Cobertura norte de España y clientes de consumo y utilities</t>
+          <t>Ya toca pharma: encaje cultural y cartera de consumo</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>ikerfel.es</t>
+          <t>moretr.com</t>
         </is>
       </c>
       <c r="N7" s="6" t="n"/>
@@ -903,12 +903,12 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Invymark</t>
+          <t>CS On Research</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Madrid (verificar)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -923,12 +923,12 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Investigación ad hoc y trackings para gran consumo y medios</t>
+          <t>Instituto 100% online con panel propio de +85.000 personas; 19 empleados; ISO 20252</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Clientes de gran consumo; complemento a DYM/Cocktail</t>
+          <t>Añade capacidad online y panel propio a Psyma</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>invymark.com</t>
+          <t>csonresearch.com</t>
         </is>
       </c>
       <c r="N8" s="6" t="n"/>
@@ -972,37 +972,37 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Netquest</t>
+          <t>Invymark</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Grupo NIQ-GfK (comprado por GfK en 2017)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Panel online de consumidores en España, Portugal y Latam</t>
+          <t>Investigación ad hoc y trackings para gran consumo y medios</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Proveedor de muestra; referencia de valoración de paneles, no disponible</t>
+          <t>Clientes de gran consumo</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>netquest.com</t>
+          <t>invymark.com</t>
         </is>
       </c>
       <c r="N9" s="6" t="n"/>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Instituto independiente líder en España; telco, electrónica de consumo, banca; +161% de crecimiento 2016-2020</t>
+          <t>Mayor instituto independiente español: telco, electrónica de consumo, banca; panel Sondea y mystery shopping</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Mayor independiente del mercado; escala y cartera telco/finanzas (ya en el deck)</t>
+          <t>Escala y cartera en telco y finanzas (ya en el deck)</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Análisis e Investigación</t>
+          <t>Gizaker</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Bilbao</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Investigación ad hoc, estudios de reputación (promotor de Merco)</t>
+          <t>Investigación social y de mercados para empresas B2B y administraciones del País Vasco</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Cartera corporativa/B2B y producto recurrente de reputación</t>
+          <t>Complemento regional a Ikerfel</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>analisiseinvestigacion.com</t>
+          <t>gizaker.com</t>
         </is>
       </c>
       <c r="N11" s="6" t="n"/>
@@ -1179,12 +1179,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Gizaker</t>
+          <t>Opinòmetre</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Bilbao</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Investigación social y de mercados, B2B y administraciones públicas del País Vasco</t>
+          <t>Investigación de mercados y opinión en Cataluña; B2B y sector público</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Complemento regional a Ikerfel; clientes institucionales</t>
+          <t>Presencia en Cataluña</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>gizaker.com</t>
+          <t>opinometre.com</t>
         </is>
       </c>
       <c r="N12" s="6" t="n"/>
@@ -1243,17 +1243,17 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Financiero / telco / B2B</t>
+          <t>Opinión y sector público</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Opinòmetre</t>
+          <t>GAD3</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1263,17 +1263,17 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Verificar en SABI</t>
+          <t>Independiente (Narciso Michavila)</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Investigación de mercados y opinión en Cataluña; B2B y sector público</t>
+          <t>Investigación social, electoral y de opinión para medios, empresas e instituciones</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Presencia en Cataluña y contratos públicos</t>
+          <t>Marca de referencia en opinión; contratos institucionales</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1283,17 +1283,17 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>opinometre.com</t>
+          <t>gad3.com</t>
         </is>
       </c>
       <c r="N13" s="6" t="n"/>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>GAD3</t>
+          <t>Sigma Dos</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1332,17 +1332,17 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Independiente (Narciso Michavila)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Investigación social, electoral y de opinión; estudios para medios y empresas</t>
+          <t>Encuestas electorales y de opinión; alianza con Dos30' para medir plataformas; socio de I+A España</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Marca de referencia en opinión; visibilidad mediática y contratos institucionales</t>
+          <t>Opinión + puente hacia audiencias (bloque 2)</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>gad3.com</t>
+          <t>sigmados.com</t>
         </is>
       </c>
       <c r="N14" s="6" t="n"/>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Sigma Dos</t>
+          <t>IMOP Insights</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Encuestas electorales y de opinión (El Mundo); alianza con Dos30' en medición de plataformas</t>
+          <t>Investigación social y de consumo; socio de I+A España</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Opinión + puente hacia audiencias (bloque 2)</t>
+          <t>Capacidad cuantitativa y contratos públicos recurrentes</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>sigmados.com</t>
+          <t>imop.es</t>
         </is>
       </c>
       <c r="N15" s="6" t="n"/>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>IMOP Insights</t>
+          <t>Celeste-Tel</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Investigación social y de consumo; trabajos de campo para organismos públicos</t>
+          <t>Encuestas de opinión y estudios de mercado; socio de I+A España</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Capacidad cuantitativa y contratos públicos recurrentes</t>
+          <t>Opinión y campo telefónico</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>imop.es</t>
+          <t>celeste-tel.es</t>
         </is>
       </c>
       <c r="N16" s="6" t="n"/>
@@ -1593,12 +1593,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>GESOP</t>
+          <t>SocioMétrica</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1613,12 +1613,12 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Estudios de opinión, sociales y electorales</t>
+          <t>Estudios sociales y de opinión; socio de I+A España</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Opinión en Cataluña; complemento a Opinòmetre</t>
+          <t>Add-on de opinión</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>gesop.net</t>
+          <t>sociometrica.es</t>
         </is>
       </c>
       <c r="N18" s="6" t="n"/>
@@ -1662,12 +1662,12 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Simple Lógica</t>
+          <t>GESOP</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1682,12 +1682,12 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Investigación social, opinión y consumo</t>
+          <t>Estudios de opinión, sociales y electorales</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Tamaño pequeño; add-on táctico</t>
+          <t>Opinión en Cataluña</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>simplelogica.com</t>
+          <t>gesop.net</t>
         </is>
       </c>
       <c r="N19" s="6" t="n"/>
@@ -1731,12 +1731,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Personality Media</t>
+          <t>Random Strategy</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Madrid / Barcelona</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1746,17 +1746,17 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Verificar en SABI</t>
+          <t>Capital español; accionistas son los propios directivos; fundada en 1989</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>Datos sindicados de notoriedad y valoración de personajes y marcas (suscripción)</t>
+          <t>Instituto con enfoque integral de investigación y consultoría; trackings y estudios continuos; ISO 20252; socio de I+A España</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>Producto de dato recurrente por suscripción: palanca del mix recurrente</t>
+          <t>Trackings continuos (ingreso recurrente) y equipo senior de consultoría</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -1771,12 +1771,12 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
         <is>
-          <t>personalitymedia.es</t>
+          <t>random-strategy.com</t>
         </is>
       </c>
       <c r="N20" s="6" t="n"/>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Ipsos Iberia</t>
+          <t>Análisis e Investigación</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -1810,32 +1810,32 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Ipsos SA (cotizada, Francia)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>Full-service; trackings de marca, CX, healthcare</t>
+          <t>Investigación y reporting de reputación corporativa (monitor Merco); socio de I+A España</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Comprador estratégico potencial de la plataforma</t>
+          <t>Producto recurrente de reputación y cartera corporativa</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="M21" s="8" t="inlineStr">
         <is>
-          <t>ipsos.com/es-es</t>
+          <t>analisiseinvestigacion.com</t>
         </is>
       </c>
       <c r="N21" s="6" t="n"/>
@@ -1869,42 +1869,42 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Kantar Insights España</t>
+          <t>Tres14 Research</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Barcelona / Madrid</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Kantar Group (Bain Capital / WPP)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>Trackings de marca (BrandZ), panel de consumo Worldpanel</t>
+          <t>Investigación de medios y eficacia publicitaria (estudio ROIMAP con Atresmedia Publicidad)</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>Comprador estratégico / benchmark de múltiplo</t>
+          <t>Tracking de notoriedad y eficacia de medios</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L22" s="8" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="M22" s="8" t="inlineStr">
         <is>
-          <t>kantar.com</t>
+          <t>tres14r.com</t>
         </is>
       </c>
       <c r="N22" s="6" t="n"/>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>YouGov España</t>
+          <t>Personality Media</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1948,32 +1948,32 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>YouGov plc (cotizada, Reino Unido)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>Panel online y BrandIndex (tracking diario de marca)</t>
+          <t>Datos sindicados de imagen de +4.000 personajes (BPM Online, por suscripción); 7 empleados en 2024</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Benchmark de tracking recurrente por suscripción</t>
+          <t>Pequeño, pero 100% dato recurrente por suscripción</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L23" s="8" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="M23" s="8" t="inlineStr">
         <is>
-          <t>business.yougov.com</t>
+          <t>personalitymedia.es</t>
         </is>
       </c>
       <c r="N23" s="6" t="n"/>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Stiga CX</t>
+          <t>IEXP · Instituto para la Experiencia del Paciente</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Madrid (verificar)</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -2027,12 +2027,12 @@
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>CX, calidad de servicio, mystery shopping y data science para +100 empresas B2B/B2C</t>
+          <t>Medición y consultoría de experiencia de paciente para hospitales (La Paz, Vall d'Hebron…) y laboratorios (Novartis, GSK, Leo Pharma)</t>
         </is>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Programas CX continuos (ingreso recurrente); extensible a experiencia de paciente</t>
+          <t>Encaje directo con el cliente pharma de Psyma y paso a medición recurrente</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="M24" s="8" t="inlineStr">
         <is>
-          <t>stigacx.com</t>
+          <t>iexp.es</t>
         </is>
       </c>
       <c r="N24" s="6" t="n"/>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>IZO</t>
+          <t>Stiga CX</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -2096,12 +2096,12 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Consultora de customer experience líder en Iberoamérica</t>
+          <t>Medición de CX, calidad de servicio, mystery shopping y data science para +100 empresas</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>CX + consultoría; abre Latam</t>
+          <t>Programas CX continuos (ingreso recurrente)</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="M25" s="8" t="inlineStr">
         <is>
-          <t>izo.es</t>
+          <t>stigacx.com</t>
         </is>
       </c>
       <c r="N25" s="6" t="n"/>
@@ -2145,12 +2145,12 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Madison MK</t>
+          <t>MDK Investigación de Mercados</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Valladolid</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -2160,27 +2160,27 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Verificar en SABI</t>
+          <t>Privada; fundada en 1998; 11-50 empleados</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>CX, insights &amp; analytics y BPO/contact center; ~40-50 M€ y 1.500-2.000 empleados</t>
+          <t>Investigación de mercados y CX; plataforma MDK Insights; oficinas en Madrid y Latam</t>
         </is>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>Demasiado grande y con peso BPO; posible socio o comprador</t>
+          <t>CX + plataforma propia; abre Latam</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L26" s="8" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="M26" s="8" t="inlineStr">
         <is>
-          <t>madisonmk.com</t>
+          <t>mdk.es</t>
         </is>
       </c>
       <c r="N26" s="6" t="n"/>
@@ -2209,12 +2209,12 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Medición de audiencias</t>
+          <t>Experiencia de cliente y paciente</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Barlovento Comunicación</t>
+          <t>Lukkap</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -2229,17 +2229,17 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>Fundador (Ricardo Vaca); sondeó el mercado en busca de comprador en 2024</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>Consultoría audiovisual: audiencias TV, social TV, big data; informes mensuales con GfK DAM</t>
+          <t>Consultoría y medición de experiencia de cliente y empleado; primer informe sectorial de experiencia de paciente en España</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>Vendedor activo; dato recurrente de audiencias; análogo a Marktest en Minerva</t>
+          <t>CX en salud (aseguradoras, laboratorios, hospitales)</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -2249,17 +2249,17 @@
       </c>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
         <is>
-          <t>barloventocomunicacion.es</t>
+          <t>lukkap.com</t>
         </is>
       </c>
       <c r="N27" s="6" t="n"/>
@@ -2278,17 +2278,17 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Medición de audiencias</t>
+          <t>Experiencia de cliente y paciente</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Dos30'</t>
+          <t>Take A Tip</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Madrid (verificar)</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -2303,12 +2303,12 @@
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Análisis de audiencias TV y plataformas; alianza con Sigma Dos para medir Netflix, Prime, Movistar+</t>
+          <t>Mystery shopping, encuestas de satisfacción y mejora continua; línea healthcare</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>Audiencias de streaming; combinable con Sigma Dos (bloque 1)</t>
+          <t>Mystery shopping en farmacia y centros sanitarios</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -2318,17 +2318,17 @@
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
         <is>
-          <t>dos30.com</t>
+          <t>takeatip.es</t>
         </is>
       </c>
       <c r="N28" s="6" t="n"/>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>GfK DAM (NIQ-GfK)</t>
+          <t>Barlovento Comunicación</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -2362,42 +2362,42 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>NIQ (Advent International)</t>
+          <t>Fundador (Ricardo Vaca); sondeó el mercado en busca de comprador en 2024</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>Medidor oficial de audiencias digitales en España desde 2022</t>
+          <t>Consultoría y reporting de audiencias TV y digitales; informes mensuales con GfK DAM</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Benchmark / comprador del bloque de medición</t>
+          <t>Vendedor activo; dato recurrente de audiencias (análogo a Marktest en Minerva)</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
         <is>
-          <t>gfkespana.es</t>
+          <t>barloventocomunicacion.es</t>
         </is>
       </c>
       <c r="N29" s="6" t="n"/>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Fifty5Blue (ex Kantar Media)</t>
+          <t>Dos30'</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -2431,42 +2431,42 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Participada por PE</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>H.I.G. Capital (compra cerrada en 2025; rebranding feb-2026)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>Medición oficial de audiencias TV en España (~5.700 hogares)</t>
+          <t>Análisis de audiencias TV y plataformas; alianza con Sigma Dos para medir Netflix, Prime y Movistar+</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>Comprador de dato y media intelligence</t>
+          <t>Audiencias de streaming; combinable con Sigma Dos (bloque 1)</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
         <is>
-          <t>kantarmedia.com</t>
+          <t>dos30.com</t>
         </is>
       </c>
       <c r="N30" s="6" t="n"/>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Comscore España</t>
+          <t>GECA</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -2500,32 +2500,32 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Filial de grupo audiovisual</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Comscore Inc. (cotizada, EE. UU.)</t>
+          <t>Grupo audiovisual (Globomedia / Grupo Imagina) — verificar</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>Medición cross-plataforma (medidor digital oficial hasta 2021)</t>
+          <t>Primera consultora española de TV (1993): audiencias, programación y contenidos</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Benchmark</t>
+          <t>Reporting de audiencias; carve-out posible</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="M31" s="8" t="inlineStr">
         <is>
-          <t>comscore.com</t>
+          <t>geca.es</t>
         </is>
       </c>
       <c r="N31" s="6" t="n"/>
@@ -2559,12 +2559,12 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Soulsight</t>
+          <t>The Cocktail Analysis</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Madrid / Barcelona</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -2574,12 +2574,12 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Verificar en SABI</t>
+          <t>Independiente (spin-off de The Cocktail)</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Consultoría de innovación, estrategia de marca e insights</t>
+          <t>Consultoría de investigación e insights: tendencias de consumo, comunicación y tecnología</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
         <is>
-          <t>soulsight.es</t>
+          <t>tcanalysis.com</t>
         </is>
       </c>
       <c r="N32" s="6" t="n"/>
@@ -2628,42 +2628,42 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Salvetti &amp; Llombart</t>
+          <t>Idea Solutions</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Madrid (verificar)</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>Participada por PE</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Minerva Insights (Ufenau), jul-2023</t>
+          <t>Fundada en 2000</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>Consultoría estratégica e insights</t>
+          <t>Investigación estratégica y cualitativa para empresas, ONG e institutos internacionales; socio de ESOMAR e I+A</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Precedente de la tesis; no disponible</t>
+          <t>Capa cualitativa-estratégica</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>Precedente (ya en Minerva)</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="M33" s="8" t="inlineStr">
         <is>
-          <t>salvetti-llombart.com</t>
+          <t>idea-solutions.net</t>
         </is>
       </c>
       <c r="N33" s="6" t="n"/>
@@ -2697,37 +2697,37 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Simon-Kucher España</t>
+          <t>Salvetti &amp; Llombart</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>Filial multinacional</t>
+          <t>Participada por PE</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>Simon-Kucher &amp; Partners (Alemania)</t>
+          <t>Minerva Insights (Ufenau), jul-2023</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>Consultoría de pricing y estrategia comercial (~31 M€ en España)</t>
+          <t>Consultoría estratégica e insights</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Benchmark de consultoría; relevante también en pharma pricing</t>
+          <t>Precedente de la tesis; no disponible</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Precedente (ya en Minerva)</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="M34" s="8" t="inlineStr">
         <is>
-          <t>simon-kucher.com</t>
+          <t>salvetti-llombart.com</t>
         </is>
       </c>
       <c r="N34" s="6" t="n"/>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>SaaS recurrente de media monitoring; base tecnológica</t>
+          <t>SaaS recurrente de media monitoring</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Epsilon Technologies</t>
+          <t>Websays</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
@@ -2855,12 +2855,12 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>Big data y analítica de redes sociales para marcas</t>
+          <t>Plataforma de social listening y reputación con PLN e IA</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Social listening con IA; complementa MyNews</t>
+          <t>Escucha social con IA para marcas y pharma</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M36" s="10" t="inlineStr">
         <is>
-          <t>epsilontec.com</t>
+          <t>websays.com</t>
         </is>
       </c>
       <c r="N36" s="6" t="n"/>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Auditmedia Group</t>
+          <t>Epsilon Technologies</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -2924,12 +2924,12 @@
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>Clipping y análisis en prensa, digital, audiovisual y redes</t>
+          <t>Big data y analítica de redes sociales para marcas</t>
         </is>
       </c>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>Consolidación del clipping</t>
+          <t>Social listening; alternativa a Websays</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="M37" s="10" t="inlineStr">
         <is>
-          <t>auditmedia.es</t>
+          <t>epsilontec.com</t>
         </is>
       </c>
       <c r="N37" s="6" t="n"/>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Seguimedia</t>
+          <t>Auditmedia Group</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -2988,17 +2988,17 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Grupo IFAT (España y Latam)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>Monitorización TV, radio, internet y redes; 6 oficinas en España</t>
+          <t>Clipping y análisis en prensa, digital, audiovisual y redes</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>Red territorial; add-on</t>
+          <t>Consolidación del clipping</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t>seguimedia.es</t>
+          <t>auditmedia.es</t>
         </is>
       </c>
       <c r="N38" s="6" t="n"/>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Hallon Consulting</t>
+          <t>Seguimedia</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -3057,17 +3057,17 @@
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>Verificar en SABI</t>
+          <t>Grupo IFAT (España y Latam)</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>Análisis de narrativas y riesgo reputacional con tecnología propia e IA</t>
+          <t>Monitorización de TV, radio, internet y redes; 6 oficinas en España</t>
         </is>
       </c>
       <c r="I39" s="10" t="inlineStr">
         <is>
-          <t>Capa analítica sobre monitorización</t>
+          <t>Red territorial; add-on</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="M39" s="10" t="inlineStr">
         <is>
-          <t>hallon.es</t>
+          <t>seguimedia.es</t>
         </is>
       </c>
       <c r="N39" s="6" t="n"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="I40" s="10" t="inlineStr">
         <is>
-          <t>Dato sindicado y recurrente de primer nivel; activo ancla del bloque</t>
+          <t>Dato sindicado y recurrente; activo ancla del bloque</t>
         </is>
       </c>
       <c r="J40" s="10" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>Control de la actividad publicitaria (ex estudio i2p con Media Hotline)</t>
+          <t>Control de actividad publicitaria (ex estudio i2p con Media Hotline)</t>
         </is>
       </c>
       <c r="I41" s="10" t="inlineStr">
@@ -3318,32 +3318,32 @@
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Graphext</t>
+          <t>ODEC</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Gandía (Valencia)</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>Participada por VC</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>VC (seed de 4,6 M$ en 2023, liderada por Hoxton Ventures)</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>Plataforma de analítica visual y modelos predictivos con IA</t>
+          <t>Tecnología para la investigación: CATI/CAWI, proceso y tabulación de datos, estudios continuos y software de planificación de medios (TOM Micro); +200 empleados; socio de I+A España</t>
         </is>
       </c>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>Herramienta de análisis para escalar proyectos</t>
+          <t>Plataforma tecnológica de proceso de datos que hoy usan los institutos; escala</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="M43" s="10" t="inlineStr">
         <is>
-          <t>graphext.com</t>
+          <t>odec.es</t>
         </is>
       </c>
       <c r="N43" s="6" t="n"/>
@@ -3387,12 +3387,12 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Bitbrain</t>
+          <t>We Are Testers</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>Zaragoza</t>
+          <t>Bilbao / Madrid</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
@@ -3402,17 +3402,17 @@
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Fundadores (spin-off Univ. Zaragoza)</t>
+          <t>Fundada en 2016</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>Neurotecnología y neuromarketing (EEG, biometría)</t>
+          <t>Plataforma de investigación y UX research con panel propio de 120.000 consumidores; socio de I+A España</t>
         </is>
       </c>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>Metodología diferencial en pharma y consumo (test de materiales y claims)</t>
+          <t>Plataforma + panel propio: pasa a Psyma a modelo tecnológico</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="M44" s="10" t="inlineStr">
         <is>
-          <t>bitbrain.com</t>
+          <t>wearetesters.com</t>
         </is>
       </c>
       <c r="N44" s="6" t="n"/>
@@ -3456,42 +3456,42 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Metricool</t>
+          <t>EncuestaFacil</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Comunidad Valenciana</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>Participada por VC</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>~5 M€ captados</t>
+          <t>Verificar en SABI</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>SaaS de analítica y gestión de redes sociales (~87 empleados)</t>
+          <t>Software de encuestas online (SaaS) para España y Latam</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>Benchmark SaaS; difícil de adquirir</t>
+          <t>Herramienta de campo online propia</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K45" s="10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L45" s="10" t="inlineStr">
@@ -3501,7 +3501,7 @@
       </c>
       <c r="M45" s="10" t="inlineStr">
         <is>
-          <t>metricool.com</t>
+          <t>encuestafacil.com</t>
         </is>
       </c>
       <c r="N45" s="6" t="n"/>
@@ -3520,12 +3520,12 @@
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Software de analítica</t>
+          <t>Insights automatizados con IA</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Typeform</t>
+          <t>Zinklar</t>
         </is>
       </c>
       <c r="E46" s="10" t="inlineStr">
@@ -3540,37 +3540,37 @@
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>VC (General Atlantic, Index…)</t>
+          <t>VC: Serie A de 5,5 M€ liderada por Caixa Capital Risc (7,6 M€ en total)</t>
         </is>
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>Software de encuestas y formularios</t>
+          <t>Plataforma de insights automatizados con IA: test de conceptos, publicidad y trackings; ~60 empleados</t>
         </is>
       </c>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>Benchmark SaaS; no adquirible</t>
+          <t>Automatiza estudios con IA; el activo más claro del bloque</t>
         </is>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>Comprador / benchmark</t>
+          <t>Target build-up</t>
         </is>
       </c>
       <c r="K46" s="10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L46" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M46" s="10" t="inlineStr">
         <is>
-          <t>typeform.com</t>
+          <t>zinklar.com</t>
         </is>
       </c>
       <c r="N46" s="6" t="n"/>
@@ -3594,17 +3594,17 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Emotion Research Lab</t>
+          <t>Sentisis</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>Independiente nacional</t>
+          <t>Participada por VC</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
@@ -3614,12 +3614,12 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Reconocimiento de emociones por IA (facial coding) para test de publicidad</t>
+          <t>Análisis con IA de opiniones de clientes y respuestas abiertas</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>Test de creatividades con IA</t>
+          <t>Codificación automática de preguntas abiertas y CX</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="M47" s="10" t="inlineStr">
         <is>
-          <t>emotionresearchlab.com</t>
+          <t>sentisis.com</t>
         </is>
       </c>
       <c r="N47" s="6" t="n"/>
@@ -3663,17 +3663,17 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Sentisis</t>
+          <t>Emotion Research Lab</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>Participada por VC</t>
+          <t>Independiente nacional</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
@@ -3683,12 +3683,12 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>Análisis de texto con IA (opiniones de clientes, CX)</t>
+          <t>IA de reconocimiento de emociones para test de publicidad</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr">
         <is>
-          <t>Codificación automática de abiertas y CX</t>
+          <t>Test de creatividades con IA</t>
         </is>
       </c>
       <c r="J48" s="10" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="K48" s="10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L48" s="10" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="M48" s="10" t="inlineStr">
         <is>
-          <t>sentisis.com</t>
+          <t>emotionresearchlab.com</t>
         </is>
       </c>
       <c r="N48" s="6" t="n"/>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>Opción tecnológica early-stage (participación minoritaria)</t>
+          <t>Opción early-stage (participación minoritaria)</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
@@ -3795,7 +3795,7 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>Fuentes: Insights + Analytics España (2024); prensa sectorial (elEconomista, Dircomfidencial, Webcapitalriesgo, Marketing Directo, Panorama Audiovisual); webs corporativas; análisis Afianza.</t>
+          <t>Criterio: solo empresas del sector insights en España (socios de I+A España o equivalentes). Fuentes: Insights + Analytics España (2024) y su directorio de empresas; prensa sectorial (elEconomista, Dircomfidencial, Webcapitalriesgo, Marketing Directo, Panorama Audiovisual); webs corporativas; análisis Afianza.</t>
         </is>
       </c>
     </row>
@@ -4346,45 +4346,45 @@
     </row>
     <row r="7">
       <c r="A7" s="21">
-        <f>'Long list'!D7</f>
+        <f>'Long list'!D10</f>
         <v/>
       </c>
       <c r="B7" s="21">
-        <f>'Long list'!H7</f>
+        <f>'Long list'!H10</f>
         <v/>
       </c>
       <c r="C7" s="21">
-        <f>IF('Long list'!N7="","[PENDIENTE]",'Long list'!N7)</f>
+        <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
         <v/>
       </c>
       <c r="D7" s="21">
-        <f>IF('Long list'!O7="","[PENDIENTE]",'Long list'!O7)</f>
+        <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
         <v/>
       </c>
       <c r="E7" s="21">
-        <f>'Long list'!I7</f>
+        <f>'Long list'!I10</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21">
-        <f>'Long list'!D10</f>
+        <f>'Long list'!D13</f>
         <v/>
       </c>
       <c r="B8" s="21">
-        <f>'Long list'!H10</f>
+        <f>'Long list'!H13</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
+        <f>IF('Long list'!N13="","[PENDIENTE]",'Long list'!N13)</f>
         <v/>
       </c>
       <c r="D8" s="21">
-        <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
+        <f>IF('Long list'!O13="","[PENDIENTE]",'Long list'!O13)</f>
         <v/>
       </c>
       <c r="E8" s="21">
-        <f>'Long list'!I10</f>
+        <f>'Long list'!I13</f>
         <v/>
       </c>
     </row>
@@ -4446,111 +4446,111 @@
     </row>
     <row r="13">
       <c r="A13" s="21">
-        <f>'Long list'!D20</f>
+        <f>'Long list'!D24</f>
         <v/>
       </c>
       <c r="B13" s="21">
-        <f>'Long list'!H20</f>
+        <f>'Long list'!H24</f>
         <v/>
       </c>
       <c r="C13" s="21">
-        <f>IF('Long list'!N20="","[PENDIENTE]",'Long list'!N20)</f>
+        <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
         <v/>
       </c>
       <c r="D13" s="21">
-        <f>IF('Long list'!O20="","[PENDIENTE]",'Long list'!O20)</f>
+        <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
         <v/>
       </c>
       <c r="E13" s="21">
-        <f>'Long list'!I20</f>
+        <f>'Long list'!I24</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21">
-        <f>'Long list'!D24</f>
+        <f>'Long list'!D25</f>
         <v/>
       </c>
       <c r="B14" s="21">
-        <f>'Long list'!H24</f>
+        <f>'Long list'!H25</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
+        <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
         <v/>
       </c>
       <c r="D14" s="21">
-        <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
+        <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
         <v/>
       </c>
       <c r="E14" s="21">
-        <f>'Long list'!I24</f>
+        <f>'Long list'!I25</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="21">
-        <f>'Long list'!D25</f>
+        <f>'Long list'!D29</f>
         <v/>
       </c>
       <c r="B15" s="21">
-        <f>'Long list'!H25</f>
+        <f>'Long list'!H29</f>
         <v/>
       </c>
       <c r="C15" s="21">
-        <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
+        <f>IF('Long list'!N29="","[PENDIENTE]",'Long list'!N29)</f>
         <v/>
       </c>
       <c r="D15" s="21">
-        <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
+        <f>IF('Long list'!O29="","[PENDIENTE]",'Long list'!O29)</f>
         <v/>
       </c>
       <c r="E15" s="21">
-        <f>'Long list'!I25</f>
+        <f>'Long list'!I29</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="21">
-        <f>'Long list'!D27</f>
+        <f>'Long list'!D30</f>
         <v/>
       </c>
       <c r="B16" s="21">
-        <f>'Long list'!H27</f>
+        <f>'Long list'!H30</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>IF('Long list'!N27="","[PENDIENTE]",'Long list'!N27)</f>
+        <f>IF('Long list'!N30="","[PENDIENTE]",'Long list'!N30)</f>
         <v/>
       </c>
       <c r="D16" s="21">
-        <f>IF('Long list'!O27="","[PENDIENTE]",'Long list'!O27)</f>
+        <f>IF('Long list'!O30="","[PENDIENTE]",'Long list'!O30)</f>
         <v/>
       </c>
       <c r="E16" s="21">
-        <f>'Long list'!I27</f>
+        <f>'Long list'!I30</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="21">
-        <f>'Long list'!D28</f>
+        <f>'Long list'!D32</f>
         <v/>
       </c>
       <c r="B17" s="21">
-        <f>'Long list'!H28</f>
+        <f>'Long list'!H32</f>
         <v/>
       </c>
       <c r="C17" s="21">
-        <f>IF('Long list'!N28="","[PENDIENTE]",'Long list'!N28)</f>
+        <f>IF('Long list'!N32="","[PENDIENTE]",'Long list'!N32)</f>
         <v/>
       </c>
       <c r="D17" s="21">
-        <f>IF('Long list'!O28="","[PENDIENTE]",'Long list'!O28)</f>
+        <f>IF('Long list'!O32="","[PENDIENTE]",'Long list'!O32)</f>
         <v/>
       </c>
       <c r="E17" s="21">
-        <f>'Long list'!I28</f>
+        <f>'Long list'!I32</f>
         <v/>
       </c>
     </row>
@@ -4612,89 +4612,89 @@
     </row>
     <row r="22">
       <c r="A22" s="21">
-        <f>'Long list'!D36</f>
+        <f>'Long list'!D40</f>
         <v/>
       </c>
       <c r="B22" s="21">
-        <f>'Long list'!H36</f>
+        <f>'Long list'!H40</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>IF('Long list'!N36="","[PENDIENTE]",'Long list'!N36)</f>
+        <f>IF('Long list'!N40="","[PENDIENTE]",'Long list'!N40)</f>
         <v/>
       </c>
       <c r="D22" s="21">
-        <f>IF('Long list'!O36="","[PENDIENTE]",'Long list'!O36)</f>
+        <f>IF('Long list'!O40="","[PENDIENTE]",'Long list'!O40)</f>
         <v/>
       </c>
       <c r="E22" s="21">
-        <f>'Long list'!I36</f>
+        <f>'Long list'!I40</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="21">
-        <f>'Long list'!D40</f>
+        <f>'Long list'!D43</f>
         <v/>
       </c>
       <c r="B23" s="21">
-        <f>'Long list'!H40</f>
+        <f>'Long list'!H43</f>
         <v/>
       </c>
       <c r="C23" s="21">
-        <f>IF('Long list'!N40="","[PENDIENTE]",'Long list'!N40)</f>
+        <f>IF('Long list'!N43="","[PENDIENTE]",'Long list'!N43)</f>
         <v/>
       </c>
       <c r="D23" s="21">
-        <f>IF('Long list'!O40="","[PENDIENTE]",'Long list'!O40)</f>
+        <f>IF('Long list'!O43="","[PENDIENTE]",'Long list'!O43)</f>
         <v/>
       </c>
       <c r="E23" s="21">
-        <f>'Long list'!I40</f>
+        <f>'Long list'!I43</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="21">
-        <f>'Long list'!D43</f>
+        <f>'Long list'!D44</f>
         <v/>
       </c>
       <c r="B24" s="21">
-        <f>'Long list'!H43</f>
+        <f>'Long list'!H44</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>IF('Long list'!N43="","[PENDIENTE]",'Long list'!N43)</f>
+        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
         <v/>
       </c>
       <c r="D24" s="21">
-        <f>IF('Long list'!O43="","[PENDIENTE]",'Long list'!O43)</f>
+        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
         <v/>
       </c>
       <c r="E24" s="21">
-        <f>'Long list'!I43</f>
+        <f>'Long list'!I44</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="21">
-        <f>'Long list'!D44</f>
+        <f>'Long list'!D46</f>
         <v/>
       </c>
       <c r="B25" s="21">
-        <f>'Long list'!H44</f>
+        <f>'Long list'!H46</f>
         <v/>
       </c>
       <c r="C25" s="21">
-        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
+        <f>IF('Long list'!N46="","[PENDIENTE]",'Long list'!N46)</f>
         <v/>
       </c>
       <c r="D25" s="21">
-        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
+        <f>IF('Long list'!O46="","[PENDIENTE]",'Long list'!O46)</f>
         <v/>
       </c>
       <c r="E25" s="21">
-        <f>'Long list'!I44</f>
+        <f>'Long list'!I46</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Tesis B: cribado de 5 empresas por vertical replicando el playbook de Minerva
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015eGgGxXjnPfmv7TgBdyPpP
</commit_message>
<xml_diff>
--- a/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
+++ b/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Long list" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Top 5 para láminas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cribado Minerva" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Top 5 para láminas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Long list'!$A$4:$Q$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cribado Minerva'!$A$11:$O$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0;(#,##0.0);-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +100,17 @@
       <color rgb="00008000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0014233C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -149,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,14 +194,33 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -196,6 +228,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DCE6F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009AAAB3"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -874,7 +920,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -1352,12 +1398,12 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -2776,12 +2822,12 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>Independiente nacional</t>
+          <t>Filial de grupo de medios</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>Verificar en SABI</t>
+          <t>Grupo La Información (Diario de Navarra) desde 2007</t>
         </is>
       </c>
       <c r="H35" s="10" t="inlineStr">
@@ -2791,22 +2837,22 @@
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>SaaS recurrente de media monitoring</t>
+          <t>Pertenece a un grupo de medios: no disponible</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>Target build-up</t>
+          <t>Comprador / benchmark</t>
         </is>
       </c>
       <c r="K35" s="10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L35" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M35" s="10" t="inlineStr">
@@ -2875,7 +2921,7 @@
       </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M36" s="10" t="inlineStr">
@@ -3343,22 +3389,22 @@
       </c>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>Plataforma tecnológica de proceso de datos que hoy usan los institutos; escala</t>
+          <t>Demasiado grande para Psyma (+200 empleados): descartada por tamaño</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>Target build-up</t>
+          <t>Comprador / benchmark</t>
         </is>
       </c>
       <c r="K43" s="10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L43" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M43" s="10" t="inlineStr">
@@ -3481,7 +3527,7 @@
       </c>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>Herramienta de campo online propia</t>
+          <t>Software de encuestas propio (equivalente a MBS en Minerva)</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
@@ -3491,12 +3537,12 @@
       </c>
       <c r="K45" s="10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L45" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M45" s="10" t="inlineStr">
@@ -3816,6 +3862,3244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cribado de targets replicando el playbook de Minerva Insights (Ufenau)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Paso 1: filtros eliminatorios (disponible y tamaño asumible; «Verificar» pasa hasta confirmar en SABI). Paso 2: puntuación 1-3 en cuatro criterios. Paso 3: las 5 mejores por vertical pasan a shortlist. Las puntuaciones son hipótesis de Afianza y el tamaño se confirma con SABI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Playbook de Minerva → equivalente para Psyma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Movimiento Minerva</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Vertical Psyma</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Equivalente buscado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>1 · Ancla de audiencias y media intelligence</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Marktest (+ Mediamonitor, Markdata, Medialog), ene-2023</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría / Tecnológicas</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Barlovento, Dos30', Websays</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>2 · Investigación sectorial</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Conecta (consumo y CX) y Amber (salud), mar-2023</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Investigación de mercados / CX y paciente</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>DYM, IO, Ikerfel, More than Research, IEXP, Stiga</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>3 · Consultoría estratégica</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Salvetti &amp; Llombart, jul-2023</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>The Cocktail Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>4 · Tecnología y dato</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Adjinn (ad intelligence con IA) y MBS (software de medios), 2025</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>InfoAdex, We Are Testers, EncuestaFacil, Zinklar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Cribado de las 45 empresas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Vertical</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Subactividad</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Equivalente en Minerva</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>F1 Disponible (sin grupo/PE)</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>F2 Tamaño asumible</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Pasa filtros</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Encaje playbook (1-3)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Recurrencia (1-3)</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Sinergia pharma/Psyma (1-3)</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Escala / señal de venta (1-3)</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Puntuación</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Ranking en vertical</t>
+        </is>
+      </c>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="O11" s="16" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Consumo y retail</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Instituto DYM</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (investigación consumo)</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G12" s="17">
+        <f>IF(AND(E12&lt;&gt;"No",F12&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="17">
+        <f>IF(G12="Sí",SUM(H12:K12),0)</f>
+        <v/>
+      </c>
+      <c r="M12" s="17">
+        <f>IF(G12="Sí",1+COUNTIFS($A$12:$A$56,A12,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L12),"—")</f>
+        <v/>
+      </c>
+      <c r="N12" s="17">
+        <f>IF(G12="No","Descartada",IF(M12&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t>Independiente con 60 años de historia; tamaño digerible</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Consumo y retail</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Ikerfel</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (investigación consumo)</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G13" s="17">
+        <f>IF(AND(E13&lt;&gt;"No",F13&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="17">
+        <f>IF(G13="Sí",SUM(H13:K13),0)</f>
+        <v/>
+      </c>
+      <c r="M13" s="17">
+        <f>IF(G13="Sí",1+COUNTIFS($A$12:$A$56,A13,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L13)+COUNTIFS($A$12:$A12,A13,$G$12:$G12,"Sí",$L$12:$L12,L13),"—")</f>
+        <v/>
+      </c>
+      <c r="N13" s="17">
+        <f>IF(G13="No","Descartada",IF(M13&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O13" s="17" t="inlineStr">
+        <is>
+          <t>Independiente; cobertura norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Consumo y retail</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>More than Research</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Amber / Conecta</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G14" s="17">
+        <f>IF(AND(E14&lt;&gt;"No",F14&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="17">
+        <f>IF(G14="Sí",SUM(H14:K14),0)</f>
+        <v/>
+      </c>
+      <c r="M14" s="17">
+        <f>IF(G14="Sí",1+COUNTIFS($A$12:$A$56,A14,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L14)+COUNTIFS($A$12:$A13,A14,$G$12:$G13,"Sí",$L$12:$L13,L14),"—")</f>
+        <v/>
+      </c>
+      <c r="N14" s="17">
+        <f>IF(G14="No","Descartada",IF(M14&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O14" s="17" t="inlineStr">
+        <is>
+          <t>Ya trabaja pharma; fundador senior</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Consumo y retail</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>CS On Research</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Conecta</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G15" s="17">
+        <f>IF(AND(E15&lt;&gt;"No",F15&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="17">
+        <f>IF(G15="Sí",SUM(H15:K15),0)</f>
+        <v/>
+      </c>
+      <c r="M15" s="17">
+        <f>IF(G15="Sí",1+COUNTIFS($A$12:$A$56,A15,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L15)+COUNTIFS($A$12:$A14,A15,$G$12:$G14,"Sí",$L$12:$L14,L15),"—")</f>
+        <v/>
+      </c>
+      <c r="N15" s="17">
+        <f>IF(G15="No","Descartada",IF(M15&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O15" s="17" t="inlineStr">
+        <is>
+          <t>Panel propio; pequeño</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Consumo y retail</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Invymark</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Conecta</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G16" s="17">
+        <f>IF(AND(E16&lt;&gt;"No",F16&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="17">
+        <f>IF(G16="Sí",SUM(H16:K16),0)</f>
+        <v/>
+      </c>
+      <c r="M16" s="17">
+        <f>IF(G16="Sí",1+COUNTIFS($A$12:$A$56,A16,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L16)+COUNTIFS($A$12:$A15,A16,$G$12:$G15,"Sí",$L$12:$L15,L16),"—")</f>
+        <v/>
+      </c>
+      <c r="N16" s="17">
+        <f>IF(G16="No","Descartada",IF(M16&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O16" s="17" t="inlineStr">
+        <is>
+          <t>Poca información pública</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Financiero / telco / B2B</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>IO Investigación</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (investigación consumo)</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G17" s="17">
+        <f>IF(AND(E17&lt;&gt;"No",F17&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H17" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" s="17">
+        <f>IF(G17="Sí",SUM(H17:K17),0)</f>
+        <v/>
+      </c>
+      <c r="M17" s="17">
+        <f>IF(G17="Sí",1+COUNTIFS($A$12:$A$56,A17,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L17)+COUNTIFS($A$12:$A16,A17,$G$12:$G16,"Sí",$L$12:$L16,L17),"—")</f>
+        <v/>
+      </c>
+      <c r="N17" s="17">
+        <f>IF(G17="No","Descartada",IF(M17&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O17" s="17" t="inlineStr">
+        <is>
+          <t>Mayor independiente; panel Sondea</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Financiero / telco / B2B</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Gizaker</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G18" s="17">
+        <f>IF(AND(E18&lt;&gt;"No",F18&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="17">
+        <f>IF(G18="Sí",SUM(H18:K18),0)</f>
+        <v/>
+      </c>
+      <c r="M18" s="17">
+        <f>IF(G18="Sí",1+COUNTIFS($A$12:$A$56,A18,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L18)+COUNTIFS($A$12:$A17,A18,$G$12:$G17,"Sí",$L$12:$L17,L18),"—")</f>
+        <v/>
+      </c>
+      <c r="N18" s="17">
+        <f>IF(G18="No","Descartada",IF(M18&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O18" s="17" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Financiero / telco / B2B</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Opinòmetre</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G19" s="17">
+        <f>IF(AND(E19&lt;&gt;"No",F19&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="17">
+        <f>IF(G19="Sí",SUM(H19:K19),0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="17">
+        <f>IF(G19="Sí",1+COUNTIFS($A$12:$A$56,A19,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L19)+COUNTIFS($A$12:$A18,A19,$G$12:$G18,"Sí",$L$12:$L18,L19),"—")</f>
+        <v/>
+      </c>
+      <c r="N19" s="17">
+        <f>IF(G19="No","Descartada",IF(M19&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O19" s="17" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>GAD3</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (investigación sectorial)</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G20" s="17">
+        <f>IF(AND(E20&lt;&gt;"No",F20&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H20" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" s="17">
+        <f>IF(G20="Sí",SUM(H20:K20),0)</f>
+        <v/>
+      </c>
+      <c r="M20" s="17">
+        <f>IF(G20="Sí",1+COUNTIFS($A$12:$A$56,A20,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L20)+COUNTIFS($A$12:$A19,A20,$G$12:$G19,"Sí",$L$12:$L19,L20),"—")</f>
+        <v/>
+      </c>
+      <c r="N20" s="17">
+        <f>IF(G20="No","Descartada",IF(M20&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O20" s="17" t="inlineStr">
+        <is>
+          <t>Marca fuerte en opinión</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Sigma Dos</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Conecta</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G21" s="17">
+        <f>IF(AND(E21&lt;&gt;"No",F21&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H21" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" s="17">
+        <f>IF(G21="Sí",SUM(H21:K21),0)</f>
+        <v/>
+      </c>
+      <c r="M21" s="17">
+        <f>IF(G21="Sí",1+COUNTIFS($A$12:$A$56,A21,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L21)+COUNTIFS($A$12:$A20,A21,$G$12:$G20,"Sí",$L$12:$L20,L21),"—")</f>
+        <v/>
+      </c>
+      <c r="N21" s="17">
+        <f>IF(G21="No","Descartada",IF(M21&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O21" s="17" t="inlineStr">
+        <is>
+          <t>Reserva: se combina con Dos30'</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>IMOP Insights</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Conecta</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G22" s="17">
+        <f>IF(AND(E22&lt;&gt;"No",F22&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H22" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" s="17">
+        <f>IF(G22="Sí",SUM(H22:K22),0)</f>
+        <v/>
+      </c>
+      <c r="M22" s="17">
+        <f>IF(G22="Sí",1+COUNTIFS($A$12:$A$56,A22,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L22)+COUNTIFS($A$12:$A21,A22,$G$12:$G21,"Sí",$L$12:$L21,L22),"—")</f>
+        <v/>
+      </c>
+      <c r="N22" s="17">
+        <f>IF(G22="No","Descartada",IF(M22&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O22" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Celeste-Tel</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G23" s="17">
+        <f>IF(AND(E23&lt;&gt;"No",F23&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="17">
+        <f>IF(G23="Sí",SUM(H23:K23),0)</f>
+        <v/>
+      </c>
+      <c r="M23" s="17">
+        <f>IF(G23="Sí",1+COUNTIFS($A$12:$A$56,A23,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L23)+COUNTIFS($A$12:$A22,A23,$G$12:$G22,"Sí",$L$12:$L22,L23),"—")</f>
+        <v/>
+      </c>
+      <c r="N23" s="17">
+        <f>IF(G23="No","Descartada",IF(M23&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O23" s="17" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>40dB.</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G24" s="17">
+        <f>IF(AND(E24&lt;&gt;"No",F24&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" s="17">
+        <f>IF(G24="Sí",SUM(H24:K24),0)</f>
+        <v/>
+      </c>
+      <c r="M24" s="17">
+        <f>IF(G24="Sí",1+COUNTIFS($A$12:$A$56,A24,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L24)+COUNTIFS($A$12:$A23,A24,$G$12:$G23,"Sí",$L$12:$L23,L24),"—")</f>
+        <v/>
+      </c>
+      <c r="N24" s="17">
+        <f>IF(G24="No","Descartada",IF(M24&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O24" s="17" t="inlineStr">
+        <is>
+          <t>Muy ligada a un cliente de medios</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>SocioMétrica</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G25" s="17">
+        <f>IF(AND(E25&lt;&gt;"No",F25&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="17">
+        <f>IF(G25="Sí",SUM(H25:K25),0)</f>
+        <v/>
+      </c>
+      <c r="M25" s="17">
+        <f>IF(G25="Sí",1+COUNTIFS($A$12:$A$56,A25,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L25)+COUNTIFS($A$12:$A24,A25,$G$12:$G24,"Sí",$L$12:$L24,L25),"—")</f>
+        <v/>
+      </c>
+      <c r="N25" s="17">
+        <f>IF(G25="No","Descartada",IF(M25&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O25" s="17" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Opinión y sector público</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>GESOP</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G26" s="17">
+        <f>IF(AND(E26&lt;&gt;"No",F26&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="17">
+        <f>IF(G26="Sí",SUM(H26:K26),0)</f>
+        <v/>
+      </c>
+      <c r="M26" s="17">
+        <f>IF(G26="Sí",1+COUNTIFS($A$12:$A$56,A26,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L26)+COUNTIFS($A$12:$A25,A26,$G$12:$G25,"Sí",$L$12:$L25,L26),"—")</f>
+        <v/>
+      </c>
+      <c r="N26" s="17">
+        <f>IF(G26="No","Descartada",IF(M26&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O26" s="17" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Trackings de marca</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Random Strategy</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (trackings)</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G27" s="17">
+        <f>IF(AND(E27&lt;&gt;"No",F27&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" s="17">
+        <f>IF(G27="Sí",SUM(H27:K27),0)</f>
+        <v/>
+      </c>
+      <c r="M27" s="17">
+        <f>IF(G27="Sí",1+COUNTIFS($A$12:$A$56,A27,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L27)+COUNTIFS($A$12:$A26,A27,$G$12:$G26,"Sí",$L$12:$L26,L27),"—")</f>
+        <v/>
+      </c>
+      <c r="N27" s="17">
+        <f>IF(G27="No","Descartada",IF(M27&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O27" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Trackings de marca</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>Análisis e Investigación</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Marktest (dato sindicado)</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G28" s="17">
+        <f>IF(AND(E28&lt;&gt;"No",F28&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H28" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I28" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" s="17">
+        <f>IF(G28="Sí",SUM(H28:K28),0)</f>
+        <v/>
+      </c>
+      <c r="M28" s="17">
+        <f>IF(G28="Sí",1+COUNTIFS($A$12:$A$56,A28,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L28)+COUNTIFS($A$12:$A27,A28,$G$12:$G27,"Sí",$L$12:$L27,L28),"—")</f>
+        <v/>
+      </c>
+      <c r="N28" s="17">
+        <f>IF(G28="No","Descartada",IF(M28&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O28" s="17" t="inlineStr">
+        <is>
+          <t>Reserva; Merco</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Trackings de marca</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Tres14 Research</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Marktest</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G29" s="17">
+        <f>IF(AND(E29&lt;&gt;"No",F29&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" s="17">
+        <f>IF(G29="Sí",SUM(H29:K29),0)</f>
+        <v/>
+      </c>
+      <c r="M29" s="17">
+        <f>IF(G29="Sí",1+COUNTIFS($A$12:$A$56,A29,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L29)+COUNTIFS($A$12:$A28,A29,$G$12:$G28,"Sí",$L$12:$L28,L29),"—")</f>
+        <v/>
+      </c>
+      <c r="N29" s="17">
+        <f>IF(G29="No","Descartada",IF(M29&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O29" s="17" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Trackings de marca</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>Personality Media</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Marktest (dato sindicado)</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G30" s="17">
+        <f>IF(AND(E30&lt;&gt;"No",F30&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H30" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" s="17">
+        <f>IF(G30="Sí",SUM(H30:K30),0)</f>
+        <v/>
+      </c>
+      <c r="M30" s="17">
+        <f>IF(G30="Sí",1+COUNTIFS($A$12:$A$56,A30,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L30)+COUNTIFS($A$12:$A29,A30,$G$12:$G29,"Sí",$L$12:$L29,L30),"—")</f>
+        <v/>
+      </c>
+      <c r="N30" s="17">
+        <f>IF(G30="No","Descartada",IF(M30&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O30" s="17" t="inlineStr">
+        <is>
+          <t>Muy pequeña (7 empleados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Experiencia de cliente y paciente</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>IEXP · Instituto para la Experiencia del Paciente</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Amber (salud) + Conecta (CX)</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G31" s="17">
+        <f>IF(AND(E31&lt;&gt;"No",F31&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H31" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" s="17">
+        <f>IF(G31="Sí",SUM(H31:K31),0)</f>
+        <v/>
+      </c>
+      <c r="M31" s="17">
+        <f>IF(G31="Sí",1+COUNTIFS($A$12:$A$56,A31,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L31)+COUNTIFS($A$12:$A30,A31,$G$12:$G30,"Sí",$L$12:$L30,L31),"—")</f>
+        <v/>
+      </c>
+      <c r="N31" s="17">
+        <f>IF(G31="No","Descartada",IF(M31&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O31" s="17" t="inlineStr">
+        <is>
+          <t>Puente directo con el cliente pharma</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Experiencia de cliente y paciente</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>Stiga CX</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (CX)</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G32" s="17">
+        <f>IF(AND(E32&lt;&gt;"No",F32&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H32" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" s="17">
+        <f>IF(G32="Sí",SUM(H32:K32),0)</f>
+        <v/>
+      </c>
+      <c r="M32" s="17">
+        <f>IF(G32="Sí",1+COUNTIFS($A$12:$A$56,A32,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L32)+COUNTIFS($A$12:$A31,A32,$G$12:$G31,"Sí",$L$12:$L31,L32),"—")</f>
+        <v/>
+      </c>
+      <c r="N32" s="17">
+        <f>IF(G32="No","Descartada",IF(M32&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O32" s="17" t="inlineStr">
+        <is>
+          <t>Programas CX continuos</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Experiencia de cliente y paciente</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>MDK Investigación de Mercados</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (CX)</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G33" s="17">
+        <f>IF(AND(E33&lt;&gt;"No",F33&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L33" s="17">
+        <f>IF(G33="Sí",SUM(H33:K33),0)</f>
+        <v/>
+      </c>
+      <c r="M33" s="17">
+        <f>IF(G33="Sí",1+COUNTIFS($A$12:$A$56,A33,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L33)+COUNTIFS($A$12:$A32,A33,$G$12:$G32,"Sí",$L$12:$L32,L33),"—")</f>
+        <v/>
+      </c>
+      <c r="N33" s="17">
+        <f>IF(G33="No","Descartada",IF(M33&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O33" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Experiencia de cliente y paciente</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Lukkap</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (CX)</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G34" s="17">
+        <f>IF(AND(E34&lt;&gt;"No",F34&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" s="17">
+        <f>IF(G34="Sí",SUM(H34:K34),0)</f>
+        <v/>
+      </c>
+      <c r="M34" s="17">
+        <f>IF(G34="Sí",1+COUNTIFS($A$12:$A$56,A34,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L34)+COUNTIFS($A$12:$A33,A34,$G$12:$G33,"Sí",$L$12:$L33,L34),"—")</f>
+        <v/>
+      </c>
+      <c r="N34" s="17">
+        <f>IF(G34="No","Descartada",IF(M34&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O34" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Experiencia de cliente y paciente</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>Take A Tip</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Conecta (CX)</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G35" s="17">
+        <f>IF(AND(E35&lt;&gt;"No",F35&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" s="17">
+        <f>IF(G35="Sí",SUM(H35:K35),0)</f>
+        <v/>
+      </c>
+      <c r="M35" s="17">
+        <f>IF(G35="Sí",1+COUNTIFS($A$12:$A$56,A35,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L35)+COUNTIFS($A$12:$A34,A35,$G$12:$G34,"Sí",$L$12:$L34,L35),"—")</f>
+        <v/>
+      </c>
+      <c r="N35" s="17">
+        <f>IF(G35="No","Descartada",IF(M35&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O35" s="17" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Medición de audiencias</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>Barlovento Comunicación</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>Marktest (audiencias, ancla)</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G36" s="17">
+        <f>IF(AND(E36&lt;&gt;"No",F36&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L36" s="17">
+        <f>IF(G36="Sí",SUM(H36:K36),0)</f>
+        <v/>
+      </c>
+      <c r="M36" s="17">
+        <f>IF(G36="Sí",1+COUNTIFS($A$12:$A$56,A36,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L36)+COUNTIFS($A$12:$A35,A36,$G$12:$G35,"Sí",$L$12:$L35,L36),"—")</f>
+        <v/>
+      </c>
+      <c r="N36" s="17">
+        <f>IF(G36="No","Descartada",IF(M36&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O36" s="17" t="inlineStr">
+        <is>
+          <t>Buscó comprador en 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Medición de audiencias</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="inlineStr">
+        <is>
+          <t>Dos30'</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>Marktest (audiencias)</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G37" s="17">
+        <f>IF(AND(E37&lt;&gt;"No",F37&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H37" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L37" s="17">
+        <f>IF(G37="Sí",SUM(H37:K37),0)</f>
+        <v/>
+      </c>
+      <c r="M37" s="17">
+        <f>IF(G37="Sí",1+COUNTIFS($A$12:$A$56,A37,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L37)+COUNTIFS($A$12:$A36,A37,$G$12:$G36,"Sí",$L$12:$L36,L37),"—")</f>
+        <v/>
+      </c>
+      <c r="N37" s="17">
+        <f>IF(G37="No","Descartada",IF(M37&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O37" s="17" t="inlineStr">
+        <is>
+          <t>Audiencias de streaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>Medición de audiencias</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>GECA</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>Marktest</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G38" s="17">
+        <f>IF(AND(E38&lt;&gt;"No",F38&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="17">
+        <f>IF(G38="Sí",SUM(H38:K38),0)</f>
+        <v/>
+      </c>
+      <c r="M38" s="17">
+        <f>IF(G38="Sí",1+COUNTIFS($A$12:$A$56,A38,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L38)+COUNTIFS($A$12:$A37,A38,$G$12:$G37,"Sí",$L$12:$L37,L38),"—")</f>
+        <v/>
+      </c>
+      <c r="N38" s="17">
+        <f>IF(G38="No","Descartada",IF(M38&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O38" s="17" t="inlineStr">
+        <is>
+          <t>Pertenece a grupo audiovisual</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Consultoría estratégica</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>The Cocktail Analysis</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>Salvetti &amp; Llombart (consultoría)</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G39" s="17">
+        <f>IF(AND(E39&lt;&gt;"No",F39&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H39" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L39" s="17">
+        <f>IF(G39="Sí",SUM(H39:K39),0)</f>
+        <v/>
+      </c>
+      <c r="M39" s="17">
+        <f>IF(G39="Sí",1+COUNTIFS($A$12:$A$56,A39,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L39)+COUNTIFS($A$12:$A38,A39,$G$12:$G38,"Sí",$L$12:$L38,L39),"—")</f>
+        <v/>
+      </c>
+      <c r="N39" s="17">
+        <f>IF(G39="No","Descartada",IF(M39&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O39" s="17" t="inlineStr">
+        <is>
+          <t>Equivalente directo a Salvetti</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>Consultoría estratégica</t>
+        </is>
+      </c>
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>Idea Solutions</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>Salvetti &amp; Llombart</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G40" s="17">
+        <f>IF(AND(E40&lt;&gt;"No",F40&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H40" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L40" s="17">
+        <f>IF(G40="Sí",SUM(H40:K40),0)</f>
+        <v/>
+      </c>
+      <c r="M40" s="17">
+        <f>IF(G40="Sí",1+COUNTIFS($A$12:$A$56,A40,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L40)+COUNTIFS($A$12:$A39,A40,$G$12:$G39,"Sí",$L$12:$L39,L40),"—")</f>
+        <v/>
+      </c>
+      <c r="N40" s="17">
+        <f>IF(G40="No","Descartada",IF(M40&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O40" s="17" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Consultoría estratégica</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>Salvetti &amp; Llombart</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>(es Minerva)</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G41" s="17">
+        <f>IF(AND(E41&lt;&gt;"No",F41&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="17">
+        <f>IF(G41="Sí",SUM(H41:K41),0)</f>
+        <v/>
+      </c>
+      <c r="M41" s="17">
+        <f>IF(G41="Sí",1+COUNTIFS($A$12:$A$56,A41,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L41)+COUNTIFS($A$12:$A40,A41,$G$12:$G40,"Sí",$L$12:$L40,L41),"—")</f>
+        <v/>
+      </c>
+      <c r="N41" s="17">
+        <f>IF(G41="No","Descartada",IF(M41&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O41" s="17" t="inlineStr">
+        <is>
+          <t>Ya comprada por Minerva</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Monitorización de medios</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>MyNews</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>Mediamonitor</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F42" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G42" s="17">
+        <f>IF(AND(E42&lt;&gt;"No",F42&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="17">
+        <f>IF(G42="Sí",SUM(H42:K42),0)</f>
+        <v/>
+      </c>
+      <c r="M42" s="17">
+        <f>IF(G42="Sí",1+COUNTIFS($A$12:$A$56,A42,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L42)+COUNTIFS($A$12:$A41,A42,$G$12:$G41,"Sí",$L$12:$L41,L42),"—")</f>
+        <v/>
+      </c>
+      <c r="N42" s="17">
+        <f>IF(G42="No","Descartada",IF(M42&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O42" s="17" t="inlineStr">
+        <is>
+          <t>Grupo La Información (Diario de Navarra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>Monitorización de medios</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>Websays</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>Mediamonitor (media intelligence)</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G43" s="17">
+        <f>IF(AND(E43&lt;&gt;"No",F43&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H43" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I43" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J43" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K43" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L43" s="17">
+        <f>IF(G43="Sí",SUM(H43:K43),0)</f>
+        <v/>
+      </c>
+      <c r="M43" s="17">
+        <f>IF(G43="Sí",1+COUNTIFS($A$12:$A$56,A43,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L43)+COUNTIFS($A$12:$A42,A43,$G$12:$G42,"Sí",$L$12:$L42,L43),"—")</f>
+        <v/>
+      </c>
+      <c r="N43" s="17">
+        <f>IF(G43="No","Descartada",IF(M43&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O43" s="17" t="inlineStr">
+        <is>
+          <t>Social listening con IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr">
+        <is>
+          <t>Monitorización de medios</t>
+        </is>
+      </c>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>Epsilon Technologies</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>Mediamonitor</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G44" s="17">
+        <f>IF(AND(E44&lt;&gt;"No",F44&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H44" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L44" s="17">
+        <f>IF(G44="Sí",SUM(H44:K44),0)</f>
+        <v/>
+      </c>
+      <c r="M44" s="17">
+        <f>IF(G44="Sí",1+COUNTIFS($A$12:$A$56,A44,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L44)+COUNTIFS($A$12:$A43,A44,$G$12:$G43,"Sí",$L$12:$L43,L44),"—")</f>
+        <v/>
+      </c>
+      <c r="N44" s="17">
+        <f>IF(G44="No","Descartada",IF(M44&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O44" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>Monitorización de medios</t>
+        </is>
+      </c>
+      <c r="C45" s="18" t="inlineStr">
+        <is>
+          <t>Auditmedia Group</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>Mediamonitor</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F45" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G45" s="17">
+        <f>IF(AND(E45&lt;&gt;"No",F45&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I45" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J45" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" s="17">
+        <f>IF(G45="Sí",SUM(H45:K45),0)</f>
+        <v/>
+      </c>
+      <c r="M45" s="17">
+        <f>IF(G45="Sí",1+COUNTIFS($A$12:$A$56,A45,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L45)+COUNTIFS($A$12:$A44,A45,$G$12:$G44,"Sí",$L$12:$L44,L45),"—")</f>
+        <v/>
+      </c>
+      <c r="N45" s="17">
+        <f>IF(G45="No","Descartada",IF(M45&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O45" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>Monitorización de medios</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr">
+        <is>
+          <t>Seguimedia</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>Mediamonitor</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F46" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G46" s="17">
+        <f>IF(AND(E46&lt;&gt;"No",F46&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="17">
+        <f>IF(G46="Sí",SUM(H46:K46),0)</f>
+        <v/>
+      </c>
+      <c r="M46" s="17">
+        <f>IF(G46="Sí",1+COUNTIFS($A$12:$A$56,A46,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L46)+COUNTIFS($A$12:$A45,A46,$G$12:$G45,"Sí",$L$12:$L45,L46),"—")</f>
+        <v/>
+      </c>
+      <c r="N46" s="17">
+        <f>IF(G46="No","Descartada",IF(M46&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O46" s="17" t="inlineStr">
+        <is>
+          <t>Pertenece al Grupo IFAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>Ad intelligence</t>
+        </is>
+      </c>
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>InfoAdex</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>Adjinn (ad intelligence)</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="G47" s="17">
+        <f>IF(AND(E47&lt;&gt;"No",F47&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H47" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L47" s="17">
+        <f>IF(G47="Sí",SUM(H47:K47),0)</f>
+        <v/>
+      </c>
+      <c r="M47" s="17">
+        <f>IF(G47="Sí",1+COUNTIFS($A$12:$A$56,A47,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L47)+COUNTIFS($A$12:$A46,A47,$G$12:$G46,"Sí",$L$12:$L46,L47),"—")</f>
+        <v/>
+      </c>
+      <c r="N47" s="17">
+        <f>IF(G47="No","Descartada",IF(M47&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O47" s="17" t="inlineStr">
+        <is>
+          <t>Accionariado y tamaño por confirmar en SABI</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>Ad intelligence</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>Arce Media</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Adjinn</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G48" s="17">
+        <f>IF(AND(E48&lt;&gt;"No",F48&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H48" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I48" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" s="17">
+        <f>IF(G48="Sí",SUM(H48:K48),0)</f>
+        <v/>
+      </c>
+      <c r="M48" s="17">
+        <f>IF(G48="Sí",1+COUNTIFS($A$12:$A$56,A48,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L48)+COUNTIFS($A$12:$A47,A48,$G$12:$G47,"Sí",$L$12:$L47,L48),"—")</f>
+        <v/>
+      </c>
+      <c r="N48" s="17">
+        <f>IF(G48="No","Descartada",IF(M48&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O48" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>Ad intelligence</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Adjinn</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>(es Minerva)</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G49" s="17">
+        <f>IF(AND(E49&lt;&gt;"No",F49&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="17">
+        <f>IF(G49="Sí",SUM(H49:K49),0)</f>
+        <v/>
+      </c>
+      <c r="M49" s="17">
+        <f>IF(G49="Sí",1+COUNTIFS($A$12:$A$56,A49,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L49)+COUNTIFS($A$12:$A48,A49,$G$12:$G48,"Sí",$L$12:$L48,L49),"—")</f>
+        <v/>
+      </c>
+      <c r="N49" s="17">
+        <f>IF(G49="No","Descartada",IF(M49&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O49" s="17" t="inlineStr">
+        <is>
+          <t>Ya comprada por Minerva</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>Software de analítica</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>ODEC</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>MBS (software de medios)</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" s="17">
+        <f>IF(AND(E50&lt;&gt;"No",F50&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="17">
+        <f>IF(G50="Sí",SUM(H50:K50),0)</f>
+        <v/>
+      </c>
+      <c r="M50" s="17">
+        <f>IF(G50="Sí",1+COUNTIFS($A$12:$A$56,A50,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L50)+COUNTIFS($A$12:$A49,A50,$G$12:$G49,"Sí",$L$12:$L49,L50),"—")</f>
+        <v/>
+      </c>
+      <c r="N50" s="17">
+        <f>IF(G50="No","Descartada",IF(M50&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O50" s="17" t="inlineStr">
+        <is>
+          <t>Demasiado grande (+200 empleados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Software de analítica</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>We Are Testers</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>MBS / Adjinn (tecnología + panel)</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G51" s="17">
+        <f>IF(AND(E51&lt;&gt;"No",F51&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H51" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I51" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J51" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L51" s="17">
+        <f>IF(G51="Sí",SUM(H51:K51),0)</f>
+        <v/>
+      </c>
+      <c r="M51" s="17">
+        <f>IF(G51="Sí",1+COUNTIFS($A$12:$A$56,A51,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L51)+COUNTIFS($A$12:$A50,A51,$G$12:$G50,"Sí",$L$12:$L50,L51),"—")</f>
+        <v/>
+      </c>
+      <c r="N51" s="17">
+        <f>IF(G51="No","Descartada",IF(M51&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O51" s="17" t="inlineStr">
+        <is>
+          <t>Plataforma + panel de 120.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Software de analítica</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>EncuestaFacil</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>MBS (software)</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G52" s="17">
+        <f>IF(AND(E52&lt;&gt;"No",F52&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H52" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I52" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L52" s="17">
+        <f>IF(G52="Sí",SUM(H52:K52),0)</f>
+        <v/>
+      </c>
+      <c r="M52" s="17">
+        <f>IF(G52="Sí",1+COUNTIFS($A$12:$A$56,A52,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L52)+COUNTIFS($A$12:$A51,A52,$G$12:$G51,"Sí",$L$12:$L51,L52),"—")</f>
+        <v/>
+      </c>
+      <c r="N52" s="17">
+        <f>IF(G52="No","Descartada",IF(M52&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O52" s="17" t="inlineStr">
+        <is>
+          <t>SaaS de encuestas; tamaño por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Insights automatizados con IA</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Zinklar</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Adjinn (IA)</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>Sí (VC)</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G53" s="17">
+        <f>IF(AND(E53&lt;&gt;"No",F53&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H53" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I53" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J53" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" s="17">
+        <f>IF(G53="Sí",SUM(H53:K53),0)</f>
+        <v/>
+      </c>
+      <c r="M53" s="17">
+        <f>IF(G53="Sí",1+COUNTIFS($A$12:$A$56,A53,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L53)+COUNTIFS($A$12:$A52,A53,$G$12:$G52,"Sí",$L$12:$L52,L53),"—")</f>
+        <v/>
+      </c>
+      <c r="N53" s="17">
+        <f>IF(G53="No","Descartada",IF(M53&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O53" s="17" t="inlineStr">
+        <is>
+          <t>Participada por VC: operación más compleja</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Insights automatizados con IA</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>Sentisis</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Adjinn (IA)</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Sí (VC)</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G54" s="17">
+        <f>IF(AND(E54&lt;&gt;"No",F54&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H54" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I54" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J54" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" s="17">
+        <f>IF(G54="Sí",SUM(H54:K54),0)</f>
+        <v/>
+      </c>
+      <c r="M54" s="17">
+        <f>IF(G54="Sí",1+COUNTIFS($A$12:$A$56,A54,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L54)+COUNTIFS($A$12:$A53,A54,$G$12:$G53,"Sí",$L$12:$L53,L54),"—")</f>
+        <v/>
+      </c>
+      <c r="N54" s="17">
+        <f>IF(G54="No","Descartada",IF(M54&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O54" s="17" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>Insights automatizados con IA</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>Emotion Research Lab</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G55" s="17">
+        <f>IF(AND(E55&lt;&gt;"No",F55&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H55" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I55" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J55" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" s="17">
+        <f>IF(G55="Sí",SUM(H55:K55),0)</f>
+        <v/>
+      </c>
+      <c r="M55" s="17">
+        <f>IF(G55="Sí",1+COUNTIFS($A$12:$A$56,A55,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L55)+COUNTIFS($A$12:$A54,A55,$G$12:$G54,"Sí",$L$12:$L54,L55),"—")</f>
+        <v/>
+      </c>
+      <c r="N55" s="17">
+        <f>IF(G55="No","Descartada",IF(M55&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O55" s="17" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>Insights automatizados con IA</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>Cuxtomers</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G56" s="17">
+        <f>IF(AND(E56&lt;&gt;"No",F56&lt;&gt;"No"),"Sí","No")</f>
+        <v/>
+      </c>
+      <c r="H56" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J56" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L56" s="17">
+        <f>IF(G56="Sí",SUM(H56:K56),0)</f>
+        <v/>
+      </c>
+      <c r="M56" s="17">
+        <f>IF(G56="Sí",1+COUNTIFS($A$12:$A$56,A56,$G$12:$G$56,"Sí",$L$12:$L$56,"&gt;"&amp;L56)+COUNTIFS($A$12:$A55,A56,$G$12:$G55,"Sí",$L$12:$L55,L56),"—")</f>
+        <v/>
+      </c>
+      <c r="N56" s="17">
+        <f>IF(G56="No","Descartada",IF(M56&lt;=5,"Shortlist","Reserva"))</f>
+        <v/>
+      </c>
+      <c r="O56" s="17" t="inlineStr">
+        <is>
+          <t>Early-stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>Embudo por vertical</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>Vertical</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="inlineStr">
+        <is>
+          <t>Universo</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>Pasan filtros</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="21" t="inlineStr">
+        <is>
+          <t>Investigación de mercados</t>
+        </is>
+      </c>
+      <c r="B60" s="21">
+        <f>COUNTIF($A$12:$A$56,A60)</f>
+        <v/>
+      </c>
+      <c r="C60" s="21">
+        <f>COUNTIFS($A$12:$A$56,A60,$G$12:$G$56,"Sí")</f>
+        <v/>
+      </c>
+      <c r="D60" s="21">
+        <f>COUNTIFS($A$12:$A$56,A60,$N$12:$N$56,"Shortlist")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="21" t="inlineStr">
+        <is>
+          <t>Reporting y consultoría</t>
+        </is>
+      </c>
+      <c r="B61" s="21">
+        <f>COUNTIF($A$12:$A$56,A61)</f>
+        <v/>
+      </c>
+      <c r="C61" s="21">
+        <f>COUNTIFS($A$12:$A$56,A61,$G$12:$G$56,"Sí")</f>
+        <v/>
+      </c>
+      <c r="D61" s="21">
+        <f>COUNTIFS($A$12:$A$56,A61,$N$12:$N$56,"Shortlist")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="21" t="inlineStr">
+        <is>
+          <t>Empresas tecnológicas</t>
+        </is>
+      </c>
+      <c r="B62" s="21">
+        <f>COUNTIF($A$12:$A$56,A62)</f>
+        <v/>
+      </c>
+      <c r="C62" s="21">
+        <f>COUNTIFS($A$12:$A$56,A62,$G$12:$G$56,"Sí")</f>
+        <v/>
+      </c>
+      <c r="D62" s="21">
+        <f>COUNTIFS($A$12:$A$56,A62,$N$12:$N$56,"Shortlist")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A11:O56"/>
+  <conditionalFormatting sqref="A12:O56">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$N12="Shortlist"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$N12="Descartada"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3828,372 +7112,372 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Resumen por bloque y subactividad</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Bloque</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>Subactividad</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="23" t="inlineStr">
         <is>
           <t>Nº empresas</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="23" t="inlineStr">
         <is>
           <t>Targets</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="23" t="inlineStr">
         <is>
           <t>Prioridad A</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="23" t="inlineStr">
         <is>
           <t>Facturación agregada (M€)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Bloque 1 · Otros sectores</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Consumo y retail</t>
         </is>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A4,'Long list'!$C$5:$C$49,B4)</f>
         <v/>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A4,'Long list'!$C$5:$C$49,B4,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A4,'Long list'!$C$5:$C$49,B4,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A4,'Long list'!$C$5:$C$49,B4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Bloque 1 · Otros sectores</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Financiero / telco / B2B</t>
         </is>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A5,'Long list'!$C$5:$C$49,B5)</f>
         <v/>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A5,'Long list'!$C$5:$C$49,B5,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A5,'Long list'!$C$5:$C$49,B5,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A5,'Long list'!$C$5:$C$49,B5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Bloque 1 · Otros sectores</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Opinión y sector público</t>
         </is>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A6,'Long list'!$C$5:$C$49,B6)</f>
         <v/>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A6,'Long list'!$C$5:$C$49,B6,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A6,'Long list'!$C$5:$C$49,B6,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A6,'Long list'!$C$5:$C$49,B6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Bloque 2 · Medición y dato recurrente</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Trackings de marca</t>
         </is>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A7,'Long list'!$C$5:$C$49,B7)</f>
         <v/>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A7,'Long list'!$C$5:$C$49,B7,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A7,'Long list'!$C$5:$C$49,B7,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A7,'Long list'!$C$5:$C$49,B7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Bloque 2 · Medición y dato recurrente</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Experiencia de cliente y paciente</t>
         </is>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A8,'Long list'!$C$5:$C$49,B8)</f>
         <v/>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A8,'Long list'!$C$5:$C$49,B8,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A8,'Long list'!$C$5:$C$49,B8,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A8,'Long list'!$C$5:$C$49,B8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Bloque 2 · Medición y dato recurrente</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Medición de audiencias</t>
         </is>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A9,'Long list'!$C$5:$C$49,B9)</f>
         <v/>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A9,'Long list'!$C$5:$C$49,B9,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A9,'Long list'!$C$5:$C$49,B9,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A9,'Long list'!$C$5:$C$49,B9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Bloque 2 · Medición y dato recurrente</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Consultoría estratégica</t>
         </is>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A10,'Long list'!$C$5:$C$49,B10)</f>
         <v/>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A10,'Long list'!$C$5:$C$49,B10,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A10,'Long list'!$C$5:$C$49,B10,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A10,'Long list'!$C$5:$C$49,B10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Bloque 3 · Tecnología e insights con IA</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Monitorización de medios</t>
         </is>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A11,'Long list'!$C$5:$C$49,B11)</f>
         <v/>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A11,'Long list'!$C$5:$C$49,B11,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A11,'Long list'!$C$5:$C$49,B11,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A11,'Long list'!$C$5:$C$49,B11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>Bloque 3 · Tecnología e insights con IA</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Ad intelligence</t>
         </is>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A12,'Long list'!$C$5:$C$49,B12)</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A12,'Long list'!$C$5:$C$49,B12,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A12,'Long list'!$C$5:$C$49,B12,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A12,'Long list'!$C$5:$C$49,B12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Bloque 3 · Tecnología e insights con IA</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Software de analítica</t>
         </is>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A13,'Long list'!$C$5:$C$49,B13)</f>
         <v/>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A13,'Long list'!$C$5:$C$49,B13,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A13,'Long list'!$C$5:$C$49,B13,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A13,'Long list'!$C$5:$C$49,B13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Bloque 3 · Tecnología e insights con IA</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Insights automatizados con IA</t>
         </is>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A14,'Long list'!$C$5:$C$49,B14)</f>
         <v/>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A14,'Long list'!$C$5:$C$49,B14,'Long list'!$J$5:$J$49,"Target build-up")</f>
         <v/>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="24">
         <f>COUNTIFS('Long list'!$B$5:$B$49,A14,'Long list'!$C$5:$C$49,B14,'Long list'!$K$5:$K$49,"A")</f>
         <v/>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="25">
         <f>SUMIFS('Long list'!$N$5:$N$49,'Long list'!$B$5:$B$49,A14,'Long list'!$C$5:$C$49,B14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n"/>
-      <c r="C15" s="17">
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="26">
         <f>SUM(C4:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="26">
         <f>SUM(D4:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="26">
         <f>SUM(E4:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="27">
         <f>SUM(F4:F14)</f>
         <v/>
       </c>
@@ -4206,34 +7490,34 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Bloque 1 · Otros sectores</t>
         </is>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="21">
         <f>COUNTIF('Long list'!$B$5:$B$49,A18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Bloque 2 · Medición y dato recurrente</t>
         </is>
       </c>
-      <c r="C19" s="19">
+      <c r="C19" s="21">
         <f>COUNTIF('Long list'!$B$5:$B$49,A19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Bloque 3 · Tecnología e insights con IA</t>
         </is>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="21">
         <f>COUNTIF('Long list'!$B$5:$B$49,A20)</f>
         <v/>
       </c>
@@ -4243,7 +7527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4260,440 +7544,440 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Cinco targets destacados por bloque (alimenta las láminas 31-33 del deck)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Bloque 1 · Otros sectores</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>Actividad</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="23" t="inlineStr">
         <is>
           <t>Facturación (M€)</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="23" t="inlineStr">
         <is>
           <t>EBITDA (M€)</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="23" t="inlineStr">
         <is>
           <t>Qué aporta a Psyma</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21">
+      <c r="A5" s="28">
         <f>'Long list'!D5</f>
         <v/>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="28">
         <f>'Long list'!H5</f>
         <v/>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="28">
         <f>IF('Long list'!N5="","[PENDIENTE]",'Long list'!N5)</f>
         <v/>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="28">
         <f>IF('Long list'!O5="","[PENDIENTE]",'Long list'!O5)</f>
         <v/>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="28">
         <f>'Long list'!I5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21">
+      <c r="A6" s="28">
         <f>'Long list'!D6</f>
         <v/>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="28">
         <f>'Long list'!H6</f>
         <v/>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="28">
         <f>IF('Long list'!N6="","[PENDIENTE]",'Long list'!N6)</f>
         <v/>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="28">
         <f>IF('Long list'!O6="","[PENDIENTE]",'Long list'!O6)</f>
         <v/>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="28">
         <f>'Long list'!I6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21">
+      <c r="A7" s="28">
+        <f>'Long list'!D7</f>
+        <v/>
+      </c>
+      <c r="B7" s="28">
+        <f>'Long list'!H7</f>
+        <v/>
+      </c>
+      <c r="C7" s="28">
+        <f>IF('Long list'!N7="","[PENDIENTE]",'Long list'!N7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="28">
+        <f>IF('Long list'!O7="","[PENDIENTE]",'Long list'!O7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="28">
+        <f>'Long list'!I7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28">
         <f>'Long list'!D10</f>
         <v/>
       </c>
-      <c r="B7" s="21">
+      <c r="B8" s="28">
         <f>'Long list'!H10</f>
         <v/>
       </c>
-      <c r="C7" s="21">
+      <c r="C8" s="28">
         <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
         <v/>
       </c>
-      <c r="D7" s="21">
+      <c r="D8" s="28">
         <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
         <v/>
       </c>
-      <c r="E7" s="21">
+      <c r="E8" s="28">
         <f>'Long list'!I10</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="21">
+    <row r="9">
+      <c r="A9" s="28">
         <f>'Long list'!D13</f>
         <v/>
       </c>
-      <c r="B8" s="21">
+      <c r="B9" s="28">
         <f>'Long list'!H13</f>
         <v/>
       </c>
-      <c r="C8" s="21">
+      <c r="C9" s="28">
         <f>IF('Long list'!N13="","[PENDIENTE]",'Long list'!N13)</f>
         <v/>
       </c>
-      <c r="D8" s="21">
+      <c r="D9" s="28">
         <f>IF('Long list'!O13="","[PENDIENTE]",'Long list'!O13)</f>
         <v/>
       </c>
-      <c r="E8" s="21">
+      <c r="E9" s="28">
         <f>'Long list'!I13</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="21">
-        <f>'Long list'!D14</f>
-        <v/>
-      </c>
-      <c r="B9" s="21">
-        <f>'Long list'!H14</f>
-        <v/>
-      </c>
-      <c r="C9" s="21">
-        <f>IF('Long list'!N14="","[PENDIENTE]",'Long list'!N14)</f>
-        <v/>
-      </c>
-      <c r="D9" s="21">
-        <f>IF('Long list'!O14="","[PENDIENTE]",'Long list'!O14)</f>
-        <v/>
-      </c>
-      <c r="E9" s="21">
-        <f>'Long list'!I14</f>
-        <v/>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Bloque 2 · Medición y dato recurrente</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Actividad</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>Facturación (M€)</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>EBITDA (M€)</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>Qué aporta a Psyma</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21">
+      <c r="A13" s="28">
         <f>'Long list'!D24</f>
         <v/>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="28">
         <f>'Long list'!H24</f>
         <v/>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="28">
         <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
         <v/>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="28">
         <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
         <v/>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="28">
         <f>'Long list'!I24</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21">
+      <c r="A14" s="28">
         <f>'Long list'!D25</f>
         <v/>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="28">
         <f>'Long list'!H25</f>
         <v/>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="28">
         <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
         <v/>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="28">
         <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
         <v/>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="28">
         <f>'Long list'!I25</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21">
+      <c r="A15" s="28">
         <f>'Long list'!D29</f>
         <v/>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="28">
         <f>'Long list'!H29</f>
         <v/>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="28">
         <f>IF('Long list'!N29="","[PENDIENTE]",'Long list'!N29)</f>
         <v/>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="28">
         <f>IF('Long list'!O29="","[PENDIENTE]",'Long list'!O29)</f>
         <v/>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="28">
         <f>'Long list'!I29</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21">
+      <c r="A16" s="28">
         <f>'Long list'!D30</f>
         <v/>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="28">
         <f>'Long list'!H30</f>
         <v/>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="28">
         <f>IF('Long list'!N30="","[PENDIENTE]",'Long list'!N30)</f>
         <v/>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="28">
         <f>IF('Long list'!O30="","[PENDIENTE]",'Long list'!O30)</f>
         <v/>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="28">
         <f>'Long list'!I30</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21">
+      <c r="A17" s="28">
         <f>'Long list'!D32</f>
         <v/>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="28">
         <f>'Long list'!H32</f>
         <v/>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="28">
         <f>IF('Long list'!N32="","[PENDIENTE]",'Long list'!N32)</f>
         <v/>
       </c>
-      <c r="D17" s="21">
+      <c r="D17" s="28">
         <f>IF('Long list'!O32="","[PENDIENTE]",'Long list'!O32)</f>
         <v/>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="28">
         <f>'Long list'!I32</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Bloque 3 · Tecnología e insights con IA</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Actividad</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Facturación (M€)</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="23" t="inlineStr">
         <is>
           <t>EBITDA (M€)</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="23" t="inlineStr">
         <is>
           <t>Qué aporta a Psyma</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21">
-        <f>'Long list'!D35</f>
-        <v/>
-      </c>
-      <c r="B21" s="21">
-        <f>'Long list'!H35</f>
-        <v/>
-      </c>
-      <c r="C21" s="21">
-        <f>IF('Long list'!N35="","[PENDIENTE]",'Long list'!N35)</f>
-        <v/>
-      </c>
-      <c r="D21" s="21">
-        <f>IF('Long list'!O35="","[PENDIENTE]",'Long list'!O35)</f>
-        <v/>
-      </c>
-      <c r="E21" s="21">
-        <f>'Long list'!I35</f>
+      <c r="A21" s="28">
+        <f>'Long list'!D36</f>
+        <v/>
+      </c>
+      <c r="B21" s="28">
+        <f>'Long list'!H36</f>
+        <v/>
+      </c>
+      <c r="C21" s="28">
+        <f>IF('Long list'!N36="","[PENDIENTE]",'Long list'!N36)</f>
+        <v/>
+      </c>
+      <c r="D21" s="28">
+        <f>IF('Long list'!O36="","[PENDIENTE]",'Long list'!O36)</f>
+        <v/>
+      </c>
+      <c r="E21" s="28">
+        <f>'Long list'!I36</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21">
+      <c r="A22" s="28">
         <f>'Long list'!D40</f>
         <v/>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="28">
         <f>'Long list'!H40</f>
         <v/>
       </c>
-      <c r="C22" s="21">
+      <c r="C22" s="28">
         <f>IF('Long list'!N40="","[PENDIENTE]",'Long list'!N40)</f>
         <v/>
       </c>
-      <c r="D22" s="21">
+      <c r="D22" s="28">
         <f>IF('Long list'!O40="","[PENDIENTE]",'Long list'!O40)</f>
         <v/>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="28">
         <f>'Long list'!I40</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21">
-        <f>'Long list'!D43</f>
-        <v/>
-      </c>
-      <c r="B23" s="21">
-        <f>'Long list'!H43</f>
-        <v/>
-      </c>
-      <c r="C23" s="21">
-        <f>IF('Long list'!N43="","[PENDIENTE]",'Long list'!N43)</f>
-        <v/>
-      </c>
-      <c r="D23" s="21">
-        <f>IF('Long list'!O43="","[PENDIENTE]",'Long list'!O43)</f>
-        <v/>
-      </c>
-      <c r="E23" s="21">
-        <f>'Long list'!I43</f>
+      <c r="A23" s="28">
+        <f>'Long list'!D44</f>
+        <v/>
+      </c>
+      <c r="B23" s="28">
+        <f>'Long list'!H44</f>
+        <v/>
+      </c>
+      <c r="C23" s="28">
+        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
+        <v/>
+      </c>
+      <c r="D23" s="28">
+        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
+        <v/>
+      </c>
+      <c r="E23" s="28">
+        <f>'Long list'!I44</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21">
-        <f>'Long list'!D44</f>
-        <v/>
-      </c>
-      <c r="B24" s="21">
-        <f>'Long list'!H44</f>
-        <v/>
-      </c>
-      <c r="C24" s="21">
-        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
-        <v/>
-      </c>
-      <c r="D24" s="21">
-        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
-        <v/>
-      </c>
-      <c r="E24" s="21">
-        <f>'Long list'!I44</f>
+      <c r="A24" s="28">
+        <f>'Long list'!D45</f>
+        <v/>
+      </c>
+      <c r="B24" s="28">
+        <f>'Long list'!H45</f>
+        <v/>
+      </c>
+      <c r="C24" s="28">
+        <f>IF('Long list'!N45="","[PENDIENTE]",'Long list'!N45)</f>
+        <v/>
+      </c>
+      <c r="D24" s="28">
+        <f>IF('Long list'!O45="","[PENDIENTE]",'Long list'!O45)</f>
+        <v/>
+      </c>
+      <c r="E24" s="28">
+        <f>'Long list'!I45</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21">
+      <c r="A25" s="28">
         <f>'Long list'!D46</f>
         <v/>
       </c>
-      <c r="B25" s="21">
+      <c r="B25" s="28">
         <f>'Long list'!H46</f>
         <v/>
       </c>
-      <c r="C25" s="21">
+      <c r="C25" s="28">
         <f>IF('Long list'!N46="","[PENDIENTE]",'Long list'!N46)</f>
         <v/>
       </c>
-      <c r="D25" s="21">
+      <c r="D25" s="28">
         <f>IF('Long list'!O46="","[PENDIENTE]",'Long list'!O46)</f>
         <v/>
       </c>
-      <c r="E25" s="21">
+      <c r="E25" s="28">
         <f>'Long list'!I46</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Tesis B: criterio add-on (fuera The Cocktail, Zinklar y Sentisis)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015eGgGxXjnPfmv7TgBdyPpP
</commit_message>
<xml_diff>
--- a/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
+++ b/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
@@ -1817,7 +1817,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -2630,22 +2630,22 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>Sube la cadena de valor: de estudio a recomendación estratégica</t>
+          <t>Demasiado grande y con perfil multinacional: no encaja como add-on</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>Target build-up</t>
+          <t>Comprador / benchmark</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>Social listening; alternativa a Websays</t>
+          <t>Social listening; complementa a Websays</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
@@ -2985,12 +2985,12 @@
       </c>
       <c r="K37" s="10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L37" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M37" s="10" t="inlineStr">
@@ -3596,22 +3596,22 @@
       </c>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>Automatiza estudios con IA; el activo más claro del bloque</t>
+          <t>Participada por VC y con operación en 80+ países: no encaja como add-on</t>
         </is>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>Target build-up</t>
+          <t>Comprador / benchmark</t>
         </is>
       </c>
       <c r="K46" s="10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L46" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M46" s="10" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Barlovento, Dos30', Websays</t>
+          <t>Barlovento, Dos30', Websays, Epsilon Technologies</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>The Cocktail Analysis</t>
+          <t>Random Strategy</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>InfoAdex, We Are Testers, EncuestaFacil, Zinklar</t>
+          <t>InfoAdex, We Are Testers, EncuestaFacil, Epsilon Technologies</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>F1 Disponible (sin grupo/PE)</t>
+          <t>F1 Add-on viable (independiente, sin grupo, multinacional ni PE/VC)</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -5078,7 +5078,7 @@
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>Conecta (trackings)</t>
+          <t>Salvetti &amp; Llombart (investigación + consultoría)</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="H27" s="19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I27" s="19" t="n">
         <v>2</v>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="O27" s="17" t="inlineStr">
         <is>
-          <t>Reserva</t>
+          <t>Capital en manos de sus directivos; investigación con enfoque de consultoría</t>
         </is>
       </c>
     </row>
@@ -5850,17 +5850,17 @@
       </c>
       <c r="D39" s="17" t="inlineStr">
         <is>
-          <t>Salvetti &amp; Llombart (consultoría)</t>
+          <t>Salvetti &amp; Llombart</t>
         </is>
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G39" s="17">
@@ -5868,16 +5868,16 @@
         <v/>
       </c>
       <c r="H39" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I39" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L39" s="17">
         <f>IF(G39="Sí",SUM(H39:K39),0)</f>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="O39" s="17" t="inlineStr">
         <is>
-          <t>Equivalente directo a Salvetti</t>
+          <t>Demasiado grande y con perfil multinacional: no encaja como add-on</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
-          <t>Mediamonitor</t>
+          <t>Mediamonitor (media intelligence)</t>
         </is>
       </c>
       <c r="E44" s="17" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="O44" s="17" t="inlineStr">
         <is>
-          <t>Reserva</t>
+          <t>Social listening; complementa a Websays</t>
         </is>
       </c>
     </row>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="E53" s="17" t="inlineStr">
         <is>
-          <t>Sí (VC)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr">
@@ -6774,16 +6774,16 @@
         <v/>
       </c>
       <c r="H53" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I53" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J53" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L53" s="17">
         <f>IF(G53="Sí",SUM(H53:K53),0)</f>
@@ -6799,7 +6799,7 @@
       </c>
       <c r="O53" s="17" t="inlineStr">
         <is>
-          <t>Participada por VC: operación más compleja</t>
+          <t>Participada por VC y con operación en 80+ países: no encaja como add-on</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="E54" s="17" t="inlineStr">
         <is>
-          <t>Sí (VC)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F54" s="17" t="inlineStr">
@@ -6839,16 +6839,16 @@
         <v/>
       </c>
       <c r="H54" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I54" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J54" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K54" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" s="17">
         <f>IF(G54="Sí",SUM(H54:K54),0)</f>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="O54" s="17" t="inlineStr">
         <is>
-          <t>Reserva</t>
+          <t>Participada por VC: no encaja como add-on</t>
         </is>
       </c>
     </row>
@@ -7730,111 +7730,111 @@
     </row>
     <row r="13">
       <c r="A13" s="28">
-        <f>'Long list'!D24</f>
+        <f>'Long list'!D20</f>
         <v/>
       </c>
       <c r="B13" s="28">
-        <f>'Long list'!H24</f>
+        <f>'Long list'!H20</f>
         <v/>
       </c>
       <c r="C13" s="28">
-        <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
+        <f>IF('Long list'!N20="","[PENDIENTE]",'Long list'!N20)</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
+        <f>IF('Long list'!O20="","[PENDIENTE]",'Long list'!O20)</f>
         <v/>
       </c>
       <c r="E13" s="28">
-        <f>'Long list'!I24</f>
+        <f>'Long list'!I20</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28">
-        <f>'Long list'!D25</f>
+        <f>'Long list'!D24</f>
         <v/>
       </c>
       <c r="B14" s="28">
-        <f>'Long list'!H25</f>
+        <f>'Long list'!H24</f>
         <v/>
       </c>
       <c r="C14" s="28">
-        <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
+        <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
+        <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
         <v/>
       </c>
       <c r="E14" s="28">
-        <f>'Long list'!I25</f>
+        <f>'Long list'!I24</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28">
-        <f>'Long list'!D29</f>
+        <f>'Long list'!D25</f>
         <v/>
       </c>
       <c r="B15" s="28">
-        <f>'Long list'!H29</f>
+        <f>'Long list'!H25</f>
         <v/>
       </c>
       <c r="C15" s="28">
-        <f>IF('Long list'!N29="","[PENDIENTE]",'Long list'!N29)</f>
+        <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>IF('Long list'!O29="","[PENDIENTE]",'Long list'!O29)</f>
+        <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
         <v/>
       </c>
       <c r="E15" s="28">
-        <f>'Long list'!I29</f>
+        <f>'Long list'!I25</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28">
-        <f>'Long list'!D30</f>
+        <f>'Long list'!D29</f>
         <v/>
       </c>
       <c r="B16" s="28">
-        <f>'Long list'!H30</f>
+        <f>'Long list'!H29</f>
         <v/>
       </c>
       <c r="C16" s="28">
-        <f>IF('Long list'!N30="","[PENDIENTE]",'Long list'!N30)</f>
+        <f>IF('Long list'!N29="","[PENDIENTE]",'Long list'!N29)</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>IF('Long list'!O30="","[PENDIENTE]",'Long list'!O30)</f>
+        <f>IF('Long list'!O29="","[PENDIENTE]",'Long list'!O29)</f>
         <v/>
       </c>
       <c r="E16" s="28">
-        <f>'Long list'!I30</f>
+        <f>'Long list'!I29</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28">
-        <f>'Long list'!D32</f>
+        <f>'Long list'!D30</f>
         <v/>
       </c>
       <c r="B17" s="28">
-        <f>'Long list'!H32</f>
+        <f>'Long list'!H30</f>
         <v/>
       </c>
       <c r="C17" s="28">
-        <f>IF('Long list'!N32="","[PENDIENTE]",'Long list'!N32)</f>
+        <f>IF('Long list'!N30="","[PENDIENTE]",'Long list'!N30)</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>IF('Long list'!O32="","[PENDIENTE]",'Long list'!O32)</f>
+        <f>IF('Long list'!O30="","[PENDIENTE]",'Long list'!O30)</f>
         <v/>
       </c>
       <c r="E17" s="28">
-        <f>'Long list'!I32</f>
+        <f>'Long list'!I30</f>
         <v/>
       </c>
     </row>
@@ -7896,89 +7896,89 @@
     </row>
     <row r="22">
       <c r="A22" s="28">
-        <f>'Long list'!D40</f>
+        <f>'Long list'!D37</f>
         <v/>
       </c>
       <c r="B22" s="28">
-        <f>'Long list'!H40</f>
+        <f>'Long list'!H37</f>
         <v/>
       </c>
       <c r="C22" s="28">
-        <f>IF('Long list'!N40="","[PENDIENTE]",'Long list'!N40)</f>
+        <f>IF('Long list'!N37="","[PENDIENTE]",'Long list'!N37)</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>IF('Long list'!O40="","[PENDIENTE]",'Long list'!O40)</f>
+        <f>IF('Long list'!O37="","[PENDIENTE]",'Long list'!O37)</f>
         <v/>
       </c>
       <c r="E22" s="28">
-        <f>'Long list'!I40</f>
+        <f>'Long list'!I37</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28">
-        <f>'Long list'!D44</f>
+        <f>'Long list'!D40</f>
         <v/>
       </c>
       <c r="B23" s="28">
-        <f>'Long list'!H44</f>
+        <f>'Long list'!H40</f>
         <v/>
       </c>
       <c r="C23" s="28">
-        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
+        <f>IF('Long list'!N40="","[PENDIENTE]",'Long list'!N40)</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
+        <f>IF('Long list'!O40="","[PENDIENTE]",'Long list'!O40)</f>
         <v/>
       </c>
       <c r="E23" s="28">
-        <f>'Long list'!I44</f>
+        <f>'Long list'!I40</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28">
-        <f>'Long list'!D45</f>
+        <f>'Long list'!D44</f>
         <v/>
       </c>
       <c r="B24" s="28">
-        <f>'Long list'!H45</f>
+        <f>'Long list'!H44</f>
         <v/>
       </c>
       <c r="C24" s="28">
-        <f>IF('Long list'!N45="","[PENDIENTE]",'Long list'!N45)</f>
+        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>IF('Long list'!O45="","[PENDIENTE]",'Long list'!O45)</f>
+        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
         <v/>
       </c>
       <c r="E24" s="28">
-        <f>'Long list'!I45</f>
+        <f>'Long list'!I44</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28">
-        <f>'Long list'!D46</f>
+        <f>'Long list'!D45</f>
         <v/>
       </c>
       <c r="B25" s="28">
-        <f>'Long list'!H46</f>
+        <f>'Long list'!H45</f>
         <v/>
       </c>
       <c r="C25" s="28">
-        <f>IF('Long list'!N46="","[PENDIENTE]",'Long list'!N46)</f>
+        <f>IF('Long list'!N45="","[PENDIENTE]",'Long list'!N45)</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>IF('Long list'!O46="","[PENDIENTE]",'Long list'!O46)</f>
+        <f>IF('Long list'!O45="","[PENDIENTE]",'Long list'!O45)</f>
         <v/>
       </c>
       <c r="E25" s="28">
-        <f>'Long list'!I46</f>
+        <f>'Long list'!I45</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Tesis B: fuera Instituto DYM (sin datos financieros), entra Sigma Dos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015eGgGxXjnPfmv7TgBdyPpP
</commit_message>
<xml_diff>
--- a/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
+++ b/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
@@ -767,7 +767,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Cartera de gran consumo y capacidad de campo; tamaño asumible para una primera compra</t>
+          <t>Sin datos financieros disponibles: fuera de la presentación</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -777,12 +777,12 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -1398,12 +1398,12 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>DYM, IO, Ikerfel, More than Research, IEXP, Stiga</t>
+          <t>IO, Ikerfel, More than Research, GAD3, Sigma Dos, IEXP, Stiga</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
@@ -4133,16 +4133,16 @@
         <v/>
       </c>
       <c r="H12" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I12" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L12" s="17">
         <f>IF(G12="Sí",SUM(H12:K12),0)</f>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="O12" s="17" t="inlineStr">
         <is>
-          <t>Independiente con 60 años de historia; tamaño digerible</t>
+          <t>Sin datos financieros disponibles: fuera de la presentación</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>Conecta</t>
+          <t>Conecta + Marktest (vía alianza con Dos30')</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
@@ -4718,7 +4718,7 @@
         <v/>
       </c>
       <c r="H21" s="19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" s="19" t="n">
         <v>1</v>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="O21" s="17" t="inlineStr">
         <is>
-          <t>Reserva: se combina con Dos30'</t>
+          <t>Alianza con Dos30' (también en shortlist): opinión + audiencias</t>
         </is>
       </c>
     </row>
@@ -7586,111 +7586,111 @@
     </row>
     <row r="5">
       <c r="A5" s="28">
-        <f>'Long list'!D5</f>
+        <f>'Long list'!D6</f>
         <v/>
       </c>
       <c r="B5" s="28">
-        <f>'Long list'!H5</f>
+        <f>'Long list'!H6</f>
         <v/>
       </c>
       <c r="C5" s="28">
-        <f>IF('Long list'!N5="","[PENDIENTE]",'Long list'!N5)</f>
+        <f>IF('Long list'!N6="","[PENDIENTE]",'Long list'!N6)</f>
         <v/>
       </c>
       <c r="D5" s="28">
-        <f>IF('Long list'!O5="","[PENDIENTE]",'Long list'!O5)</f>
+        <f>IF('Long list'!O6="","[PENDIENTE]",'Long list'!O6)</f>
         <v/>
       </c>
       <c r="E5" s="28">
-        <f>'Long list'!I5</f>
+        <f>'Long list'!I6</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="28">
-        <f>'Long list'!D6</f>
+        <f>'Long list'!D7</f>
         <v/>
       </c>
       <c r="B6" s="28">
-        <f>'Long list'!H6</f>
+        <f>'Long list'!H7</f>
         <v/>
       </c>
       <c r="C6" s="28">
-        <f>IF('Long list'!N6="","[PENDIENTE]",'Long list'!N6)</f>
+        <f>IF('Long list'!N7="","[PENDIENTE]",'Long list'!N7)</f>
         <v/>
       </c>
       <c r="D6" s="28">
-        <f>IF('Long list'!O6="","[PENDIENTE]",'Long list'!O6)</f>
+        <f>IF('Long list'!O7="","[PENDIENTE]",'Long list'!O7)</f>
         <v/>
       </c>
       <c r="E6" s="28">
-        <f>'Long list'!I6</f>
+        <f>'Long list'!I7</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="28">
-        <f>'Long list'!D7</f>
+        <f>'Long list'!D10</f>
         <v/>
       </c>
       <c r="B7" s="28">
-        <f>'Long list'!H7</f>
+        <f>'Long list'!H10</f>
         <v/>
       </c>
       <c r="C7" s="28">
-        <f>IF('Long list'!N7="","[PENDIENTE]",'Long list'!N7)</f>
+        <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
         <v/>
       </c>
       <c r="D7" s="28">
-        <f>IF('Long list'!O7="","[PENDIENTE]",'Long list'!O7)</f>
+        <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
         <v/>
       </c>
       <c r="E7" s="28">
-        <f>'Long list'!I7</f>
+        <f>'Long list'!I10</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="28">
-        <f>'Long list'!D10</f>
+        <f>'Long list'!D13</f>
         <v/>
       </c>
       <c r="B8" s="28">
-        <f>'Long list'!H10</f>
+        <f>'Long list'!H13</f>
         <v/>
       </c>
       <c r="C8" s="28">
-        <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
+        <f>IF('Long list'!N13="","[PENDIENTE]",'Long list'!N13)</f>
         <v/>
       </c>
       <c r="D8" s="28">
-        <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
+        <f>IF('Long list'!O13="","[PENDIENTE]",'Long list'!O13)</f>
         <v/>
       </c>
       <c r="E8" s="28">
-        <f>'Long list'!I10</f>
+        <f>'Long list'!I13</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="28">
-        <f>'Long list'!D13</f>
+        <f>'Long list'!D14</f>
         <v/>
       </c>
       <c r="B9" s="28">
-        <f>'Long list'!H13</f>
+        <f>'Long list'!H14</f>
         <v/>
       </c>
       <c r="C9" s="28">
-        <f>IF('Long list'!N13="","[PENDIENTE]",'Long list'!N13)</f>
+        <f>IF('Long list'!N14="","[PENDIENTE]",'Long list'!N14)</f>
         <v/>
       </c>
       <c r="D9" s="28">
-        <f>IF('Long list'!O13="","[PENDIENTE]",'Long list'!O13)</f>
+        <f>IF('Long list'!O14="","[PENDIENTE]",'Long list'!O14)</f>
         <v/>
       </c>
       <c r="E9" s="28">
-        <f>'Long list'!I13</f>
+        <f>'Long list'!I14</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Tesis B: fuera More than Research, EncuestaFacil, Barlovento y Websays por tamaño y falta de datos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015eGgGxXjnPfmv7TgBdyPpP
</commit_message>
<xml_diff>
--- a/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
+++ b/tesis_b/Psyma_TesisB_longlist_ESOMAR.xlsx
@@ -905,7 +905,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Ya toca pharma: encaje cultural y cartera de consumo</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Añade capacidad online y panel propio a Psyma</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Vendedor activo; dato recurrente de audiencias (análogo a Marktest en Minerva)</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Escucha social con IA para marcas y pharma</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
@@ -2916,12 +2916,12 @@
       </c>
       <c r="K36" s="10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M36" s="10" t="inlineStr">
@@ -3054,12 +3054,12 @@
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L38" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M38" s="10" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="K41" s="10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L41" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M41" s="10" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>Software de encuestas propio (equivalente a MBS en Minerva)</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
@@ -3537,12 +3537,12 @@
       </c>
       <c r="K45" s="10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L45" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M45" s="10" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Barlovento, Dos30', Websays, Epsilon Technologies</t>
+          <t>Dos30', Epsilon Technologies, Auditmedia</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>IO, Ikerfel, More than Research, GAD3, Sigma Dos, IEXP, Stiga</t>
+          <t>IO, Ikerfel, GAD3, Sigma Dos, IMOP, IEXP, Stiga</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>InfoAdex, We Are Testers, EncuestaFacil, Epsilon Technologies</t>
+          <t>InfoAdex, Arce Media, We Are Testers</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G14" s="17">
@@ -4263,16 +4263,16 @@
         <v/>
       </c>
       <c r="H14" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I14" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L14" s="17">
         <f>IF(G14="Sí",SUM(H14:K14),0)</f>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="O14" s="17" t="inlineStr">
         <is>
-          <t>Ya trabaja pharma; fundador senior</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
     </row>
@@ -4320,7 +4320,7 @@
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G15" s="17">
@@ -4328,16 +4328,16 @@
         <v/>
       </c>
       <c r="H15" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I15" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="17">
         <f>IF(G15="Sí",SUM(H15:K15),0)</f>
@@ -4353,7 +4353,7 @@
       </c>
       <c r="O15" s="17" t="inlineStr">
         <is>
-          <t>Panel propio; pequeño</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G36" s="17">
@@ -5673,16 +5673,16 @@
         <v/>
       </c>
       <c r="H36" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I36" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J36" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L36" s="17">
         <f>IF(G36="Sí",SUM(H36:K36),0)</f>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="O36" s="17" t="inlineStr">
         <is>
-          <t>Buscó comprador en 2024</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G43" s="17">
@@ -6124,16 +6124,16 @@
         <v/>
       </c>
       <c r="H43" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I43" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J43" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L43" s="17">
         <f>IF(G43="Sí",SUM(H43:K43),0)</f>
@@ -6149,7 +6149,7 @@
       </c>
       <c r="O43" s="17" t="inlineStr">
         <is>
-          <t>Social listening con IA</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G52" s="17">
@@ -6709,16 +6709,16 @@
         <v/>
       </c>
       <c r="H52" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I52" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J52" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" s="19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L52" s="17">
         <f>IF(G52="Sí",SUM(H52:K52),0)</f>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="O52" s="17" t="inlineStr">
         <is>
-          <t>SaaS de encuestas; tamaño por confirmar</t>
+          <t>Tamaño reducido y sin datos financieros suficientes: fuera de la presentación</t>
         </is>
       </c>
     </row>
@@ -7608,89 +7608,89 @@
     </row>
     <row r="6">
       <c r="A6" s="28">
-        <f>'Long list'!D7</f>
+        <f>'Long list'!D10</f>
         <v/>
       </c>
       <c r="B6" s="28">
-        <f>'Long list'!H7</f>
+        <f>'Long list'!H10</f>
         <v/>
       </c>
       <c r="C6" s="28">
-        <f>IF('Long list'!N7="","[PENDIENTE]",'Long list'!N7)</f>
+        <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
         <v/>
       </c>
       <c r="D6" s="28">
-        <f>IF('Long list'!O7="","[PENDIENTE]",'Long list'!O7)</f>
+        <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
         <v/>
       </c>
       <c r="E6" s="28">
-        <f>'Long list'!I7</f>
+        <f>'Long list'!I10</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="28">
-        <f>'Long list'!D10</f>
+        <f>'Long list'!D13</f>
         <v/>
       </c>
       <c r="B7" s="28">
-        <f>'Long list'!H10</f>
+        <f>'Long list'!H13</f>
         <v/>
       </c>
       <c r="C7" s="28">
-        <f>IF('Long list'!N10="","[PENDIENTE]",'Long list'!N10)</f>
+        <f>IF('Long list'!N13="","[PENDIENTE]",'Long list'!N13)</f>
         <v/>
       </c>
       <c r="D7" s="28">
-        <f>IF('Long list'!O10="","[PENDIENTE]",'Long list'!O10)</f>
+        <f>IF('Long list'!O13="","[PENDIENTE]",'Long list'!O13)</f>
         <v/>
       </c>
       <c r="E7" s="28">
-        <f>'Long list'!I10</f>
+        <f>'Long list'!I13</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="28">
-        <f>'Long list'!D13</f>
+        <f>'Long list'!D14</f>
         <v/>
       </c>
       <c r="B8" s="28">
-        <f>'Long list'!H13</f>
+        <f>'Long list'!H14</f>
         <v/>
       </c>
       <c r="C8" s="28">
-        <f>IF('Long list'!N13="","[PENDIENTE]",'Long list'!N13)</f>
+        <f>IF('Long list'!N14="","[PENDIENTE]",'Long list'!N14)</f>
         <v/>
       </c>
       <c r="D8" s="28">
-        <f>IF('Long list'!O13="","[PENDIENTE]",'Long list'!O13)</f>
+        <f>IF('Long list'!O14="","[PENDIENTE]",'Long list'!O14)</f>
         <v/>
       </c>
       <c r="E8" s="28">
-        <f>'Long list'!I13</f>
+        <f>'Long list'!I14</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="28">
-        <f>'Long list'!D14</f>
+        <f>'Long list'!D15</f>
         <v/>
       </c>
       <c r="B9" s="28">
-        <f>'Long list'!H14</f>
+        <f>'Long list'!H15</f>
         <v/>
       </c>
       <c r="C9" s="28">
-        <f>IF('Long list'!N14="","[PENDIENTE]",'Long list'!N14)</f>
+        <f>IF('Long list'!N15="","[PENDIENTE]",'Long list'!N15)</f>
         <v/>
       </c>
       <c r="D9" s="28">
-        <f>IF('Long list'!O14="","[PENDIENTE]",'Long list'!O14)</f>
+        <f>IF('Long list'!O15="","[PENDIENTE]",'Long list'!O15)</f>
         <v/>
       </c>
       <c r="E9" s="28">
-        <f>'Long list'!I14</f>
+        <f>'Long list'!I15</f>
         <v/>
       </c>
     </row>
@@ -7752,67 +7752,67 @@
     </row>
     <row r="14">
       <c r="A14" s="28">
-        <f>'Long list'!D24</f>
+        <f>'Long list'!D21</f>
         <v/>
       </c>
       <c r="B14" s="28">
-        <f>'Long list'!H24</f>
+        <f>'Long list'!H21</f>
         <v/>
       </c>
       <c r="C14" s="28">
-        <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
+        <f>IF('Long list'!N21="","[PENDIENTE]",'Long list'!N21)</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
+        <f>IF('Long list'!O21="","[PENDIENTE]",'Long list'!O21)</f>
         <v/>
       </c>
       <c r="E14" s="28">
-        <f>'Long list'!I24</f>
+        <f>'Long list'!I21</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28">
-        <f>'Long list'!D25</f>
+        <f>'Long list'!D24</f>
         <v/>
       </c>
       <c r="B15" s="28">
-        <f>'Long list'!H25</f>
+        <f>'Long list'!H24</f>
         <v/>
       </c>
       <c r="C15" s="28">
-        <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
+        <f>IF('Long list'!N24="","[PENDIENTE]",'Long list'!N24)</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
+        <f>IF('Long list'!O24="","[PENDIENTE]",'Long list'!O24)</f>
         <v/>
       </c>
       <c r="E15" s="28">
-        <f>'Long list'!I25</f>
+        <f>'Long list'!I24</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28">
-        <f>'Long list'!D29</f>
+        <f>'Long list'!D25</f>
         <v/>
       </c>
       <c r="B16" s="28">
-        <f>'Long list'!H29</f>
+        <f>'Long list'!H25</f>
         <v/>
       </c>
       <c r="C16" s="28">
-        <f>IF('Long list'!N29="","[PENDIENTE]",'Long list'!N29)</f>
+        <f>IF('Long list'!N25="","[PENDIENTE]",'Long list'!N25)</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>IF('Long list'!O29="","[PENDIENTE]",'Long list'!O29)</f>
+        <f>IF('Long list'!O25="","[PENDIENTE]",'Long list'!O25)</f>
         <v/>
       </c>
       <c r="E16" s="28">
-        <f>'Long list'!I29</f>
+        <f>'Long list'!I25</f>
         <v/>
       </c>
     </row>
@@ -7874,45 +7874,45 @@
     </row>
     <row r="21">
       <c r="A21" s="28">
-        <f>'Long list'!D36</f>
+        <f>'Long list'!D37</f>
         <v/>
       </c>
       <c r="B21" s="28">
-        <f>'Long list'!H36</f>
+        <f>'Long list'!H37</f>
         <v/>
       </c>
       <c r="C21" s="28">
-        <f>IF('Long list'!N36="","[PENDIENTE]",'Long list'!N36)</f>
+        <f>IF('Long list'!N37="","[PENDIENTE]",'Long list'!N37)</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>IF('Long list'!O36="","[PENDIENTE]",'Long list'!O36)</f>
+        <f>IF('Long list'!O37="","[PENDIENTE]",'Long list'!O37)</f>
         <v/>
       </c>
       <c r="E21" s="28">
-        <f>'Long list'!I36</f>
+        <f>'Long list'!I37</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28">
-        <f>'Long list'!D37</f>
+        <f>'Long list'!D38</f>
         <v/>
       </c>
       <c r="B22" s="28">
-        <f>'Long list'!H37</f>
+        <f>'Long list'!H38</f>
         <v/>
       </c>
       <c r="C22" s="28">
-        <f>IF('Long list'!N37="","[PENDIENTE]",'Long list'!N37)</f>
+        <f>IF('Long list'!N38="","[PENDIENTE]",'Long list'!N38)</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>IF('Long list'!O37="","[PENDIENTE]",'Long list'!O37)</f>
+        <f>IF('Long list'!O38="","[PENDIENTE]",'Long list'!O38)</f>
         <v/>
       </c>
       <c r="E22" s="28">
-        <f>'Long list'!I37</f>
+        <f>'Long list'!I38</f>
         <v/>
       </c>
     </row>
@@ -7940,45 +7940,45 @@
     </row>
     <row r="24">
       <c r="A24" s="28">
-        <f>'Long list'!D44</f>
+        <f>'Long list'!D41</f>
         <v/>
       </c>
       <c r="B24" s="28">
-        <f>'Long list'!H44</f>
+        <f>'Long list'!H41</f>
         <v/>
       </c>
       <c r="C24" s="28">
-        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
+        <f>IF('Long list'!N41="","[PENDIENTE]",'Long list'!N41)</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
+        <f>IF('Long list'!O41="","[PENDIENTE]",'Long list'!O41)</f>
         <v/>
       </c>
       <c r="E24" s="28">
-        <f>'Long list'!I44</f>
+        <f>'Long list'!I41</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28">
-        <f>'Long list'!D45</f>
+        <f>'Long list'!D44</f>
         <v/>
       </c>
       <c r="B25" s="28">
-        <f>'Long list'!H45</f>
+        <f>'Long list'!H44</f>
         <v/>
       </c>
       <c r="C25" s="28">
-        <f>IF('Long list'!N45="","[PENDIENTE]",'Long list'!N45)</f>
+        <f>IF('Long list'!N44="","[PENDIENTE]",'Long list'!N44)</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>IF('Long list'!O45="","[PENDIENTE]",'Long list'!O45)</f>
+        <f>IF('Long list'!O44="","[PENDIENTE]",'Long list'!O44)</f>
         <v/>
       </c>
       <c r="E25" s="28">
-        <f>'Long list'!I45</f>
+        <f>'Long list'!I44</f>
         <v/>
       </c>
     </row>

</xml_diff>